<commit_message>
Shared email with same surname = same person (warn, merged at export)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHXVUB5nxWZdDwRJd5MuyH
</commit_message>
<xml_diff>
--- a/data/export/batch1.xlsx
+++ b/data/export/batch1.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X63"/>
+  <dimension ref="A1:X64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5592,27 +5592,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Duke University</t>
+          <t>Boston University</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Biomedical Engineering</t>
+          <t>Psychological &amp; Brain Sciences; Graduate Program for Neuroscience (faculty); Center for Systems Neuroscience</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Junjie Yao</t>
+          <t>Arthur Lee</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Jeffrey N. Vinik Associate Professor of Biomedical Engineering</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5622,48 +5622,44 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>medical-AI</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Photoacoustic tomography technology and image reconstruction for functional brain imaging and cancer.</t>
+          <t>Card has no research text or papers.</t>
         </is>
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>junjie.yao@duke.edu</t>
+          <t>artlee@bu.edu</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>https://bme.duke.edu/people/junjie-yao/</t>
+          <t>https://www.bu.edu/psych/profile/arthur-sangil-lee/</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>https://photoacoustics.pratt.duke.edu/</t>
+          <t>http://thedecodinglab.com/</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>“Three-dimensional photoacoustic tomography with ultrasound localization priors.” Photoacoustics 51 (October 2026)</t>
+          <t>Neural decoders: saving the baby from the bathwater</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>“Noninvasive whole-brain imaging of glymphatic dynamics.” Sci Adv 12, no. 25 (June 19, 2026)</t>
-        </is>
-      </c>
-      <c r="P52" t="inlineStr">
-        <is>
-          <t>Flexible ultrasound array for subcortical brain stimulation in humans: a simulation study (2026) | Hepatocyte hedgehog signaling controls ferroptosis to alleviate aging-related organ dysfunction (2026)</t>
-        </is>
-      </c>
+          <t>Distinguishing deception from its confounds by improving the validity of fMRI-based neural prediction</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr"/>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>https://bme.duke.edu/people/page/3/?group=faculty</t>
+          <t>https://www.bu.edu/psych/people/faculty/</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -5673,20 +5669,28 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>Yes: There are typically 1-2 openings for graduate students each year. Candidates should apply to the Biomedical Engineering Department and specify interest in working with Dr. Yao</t>
+          <t>Yes: We are looking for Ph.D. students interested in our research.</t>
         </is>
       </c>
       <c r="T52" t="inlineStr"/>
-      <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Please feel free to send an email to Arthur (see contact) to let him know to look out for your application.</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>His interest in validating neural decoders (confounds, interpretability) connects to the EEG motor-imagery decoder with run-grouped validation.</t>
+        </is>
+      </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>imaging hardware/optics lab, ML is secondary; associate professor; start year not found (lab 'Founded in 2016')</t>
+          <t>psychology department; applications go through Psychology or Neuroscience program, not CS/Stats</t>
         </is>
       </c>
       <c r="X52" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; dossier reader says C: Downgraded B-&gt;C: lab builds photoacoustic/ultrasound systems; computational work is a minor part and no applicant projec</t>
+          <t>also listed as Arthur Sangil Lee</t>
         </is>
       </c>
     </row>
@@ -5701,17 +5705,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Biostatistics &amp; Bioinformatics (SOM)</t>
+          <t>Biomedical Engineering</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Lin Lin</t>
+          <t>Junjie Yao</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Associate Professor of Biostatistics &amp; Bioinformatics</t>
+          <t>Jeffrey N. Vinik Associate Professor of Biomedical Engineering</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -5731,39 +5735,43 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Cytometry-based outcome prediction (cytoGPNet) alongside transplant and lung cancer immune studies.</t>
+          <t>Photoacoustic tomography technology and image reconstruction for functional brain imaging and cancer.</t>
         </is>
       </c>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>lynn.lin@duke.edu</t>
+          <t>junjie.yao@duke.edu</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/lin-lin</t>
+          <t>https://bme.duke.edu/people/junjie-yao/</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/lin-lin</t>
+          <t>https://photoacoustics.pratt.duke.edu/</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>cytoGPNet: Enhancing clinical outcome prediction accuracy using longitudinal cytometry data in small cohort studies</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr"/>
+          <t>“Three-dimensional photoacoustic tomography with ultrasound localization priors.” Photoacoustics 51 (October 2026)</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>“Noninvasive whole-brain imaging of glymphatic dynamics.” Sci Adv 12, no. 25 (June 19, 2026)</t>
+        </is>
+      </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>CD154 blockade effectively controls antibody-mediated rejection in highly sensitized nonhuman primate kidney transplant recipients (2025) | Perioperative pembrolizumab in early-stage non-small cell lung cancer (NSCLC): conventional and distribution-based immune profiling of the tumor microenvironment and peripheral circulation (2025)</t>
+          <t>Flexible ultrasound array for subcortical brain stimulation in humans: a simulation study (2026) | Hepatocyte hedgehog signaling controls ferroptosis to alleviate aging-related organ dysfunction (2026)</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/people/faculty?page=3</t>
+          <t>https://bme.duke.edu/people/page/3/?group=faculty</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -5773,24 +5781,20 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unspecified: </t>
+          <t>Yes: There are typically 1-2 openings for graduate students each year. Candidates should apply to the Biomedical Engineering Department and specify interest in working with Dr. Yao</t>
         </is>
       </c>
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
-      <c r="V53" t="inlineStr">
-        <is>
-          <t>Her cytoGPNet work on prediction in small cohorts relates to the applicant's leakage-aware, multi-seed evaluation of the arborphy fusion model.</t>
-        </is>
-      </c>
+      <c r="V53" t="inlineStr"/>
       <c r="W53" t="inlineStr">
         <is>
-          <t>no lab site found (1 search + 1 targeted); paper page is a journal article, not her own publications page; associate professor; promotion year not found; recruiting info not found</t>
+          <t>imaging hardware/optics lab, ML is secondary; associate professor; start year not found (lab 'Founded in 2016')</t>
         </is>
       </c>
       <c r="X53" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's</t>
+          <t>associate: confirm promoted 2020+; dossier reader says C: Downgraded B-&gt;C: lab builds photoacoustic/ultrasound systems; computational work is a minor part and no applicant projec</t>
         </is>
       </c>
     </row>
@@ -5810,17 +5814,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Pan Xu</t>
+          <t>Lin Lin</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Assistant Professor of Biostatistics &amp; Bioinformatics</t>
+          <t>Associate Professor of Biostatistics &amp; Bioinformatics</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -5835,43 +5839,39 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Reinforcement learning for decision support in ECMO management.</t>
+          <t>Cytometry-based outcome prediction (cytoGPNet) alongside transplant and lung cancer immune studies.</t>
         </is>
       </c>
       <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>pan.xu@duke.edu</t>
+          <t>lynn.lin@duke.edu</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/pan-xu</t>
+          <t>https://biostat.duke.edu/profile/lin-lin</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>https://panxulab.github.io/</t>
+          <t>https://biostat.duke.edu/profile/lin-lin</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Extremely Sparse Supervision Incentivizes Reasoning Ability</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>Decoupled Marginal Sharpening for Training-Free Inference-Time Scaling</t>
-        </is>
-      </c>
+          <t>cytoGPNet: Enhancing clinical outcome prediction accuracy using longitudinal cytometry data in small cohort studies</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
         <is>
-          <t>rECMOmender: Reinforcement Learning for Decision Support in Venovenous Extracorporeal Membrane Oxygenation Management (2026)</t>
+          <t>CD154 blockade effectively controls antibody-mediated rejection in highly sensitized nonhuman primate kidney transplant recipients (2025) | Perioperative pembrolizumab in early-stage non-small cell lung cancer (NSCLC): conventional and distribution-based immune profiling of the tumor microenvironment and peripheral circulation (2025)</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/people/faculty?page=6</t>
+          <t>https://biostat.duke.edu/people/faculty?page=3</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5881,24 +5881,24 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yes: I am always happy to collaborate with highly motivated and self-driven students who are genuinely interested in our research. Before contacting me, please take the time to carefully read at least one </t>
+          <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
       <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="inlineStr">
         <is>
-          <t>His 'Extremely Sparse Supervision' paper runs on-policy distillation experiments on the Qwen3 family, which touches the applicant's Qwen3 probing/steering interp work (evaluation-focused, not a causal claim).</t>
+          <t>Her cytoGPNet work on prediction in small cohorts relates to the applicant's leakage-aware, multi-seed evaluation of the arborphy fusion model.</t>
         </is>
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>site requires reading a lab paper and a specific 5-8 sentence note (CV + which paper/why/background) before he replies; start year not stated; original panxu-ai.github.io redirects to panxulab.github.io</t>
+          <t>no lab site found (1 search + 1 targeted); paper page is a journal article, not her own publications page; associate professor; promotion year not found; recruiting info not found</t>
         </is>
       </c>
       <c r="X54" t="inlineStr">
         <is>
-          <t>dossier reader says A: Upgraded B-&gt;A: ML-core (RL, LLMs, data-efficient learning), tenure-track assistant professor with healthcare application</t>
+          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's</t>
         </is>
       </c>
     </row>
@@ -5913,12 +5913,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Biostatistics &amp; Bioinformatics (SOM); CBB program</t>
+          <t>Biostatistics &amp; Bioinformatics (SOM)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Pixu Shi</t>
+          <t>Pan Xu</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -5938,40 +5938,48 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>AI-for-science</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Trajectory-guided dimensionality reduction for multi-sample single-cell RNA-seq data.</t>
+          <t>Reinforcement learning for decision support in ECMO management.</t>
         </is>
       </c>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>pixu.shi@duke.edu</t>
+          <t>pan.xu@duke.edu</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/pixu-shi</t>
+          <t>https://biostat.duke.edu/profile/pan-xu</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/pixu-shi</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
-      <c r="O55" t="inlineStr"/>
+          <t>https://panxulab.github.io/</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Extremely Sparse Supervision Incentivizes Reasoning Ability</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Decoupled Marginal Sharpening for Training-Free Inference-Time Scaling</t>
+        </is>
+      </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Branched chain amino acid metabolism and microbiome in adolescents with obesity during weight loss therapy (2026) | Characterizing the composition and diversity of the vaginal microbiome in ovarian cancer (2026)</t>
+          <t>rECMOmender: Reinforcement Learning for Decision Support in Venovenous Extracorporeal Membrane Oxygenation Management (2026)</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/people/faculty?page=5</t>
+          <t>https://biostat.duke.edu/people/faculty?page=6</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5981,20 +5989,24 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unspecified: </t>
+          <t xml:space="preserve">Yes: I am always happy to collaborate with highly motivated and self-driven students who are genuinely interested in our research. Before contacting me, please take the time to carefully read at least one </t>
         </is>
       </c>
       <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr"/>
-      <c r="V55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>His 'Extremely Sparse Supervision' paper runs on-policy distillation experiments on the Qwen3 family, which touches the applicant's Qwen3 probing/steering interp work (evaluation-focused, not a causal claim).</t>
+        </is>
+      </c>
       <c r="W55" t="inlineStr">
         <is>
-          <t>no lab/personal site found (1 search); official profile has no research text; her 2026 Bioinformatics paper is listed only on Wenpin Hou's page, not hers, so not recorded as paper; recruiting info not found</t>
+          <t>site requires reading a lab paper and a specific 5-8 sentence note (CV + which paper/why/background) before he replies; start year not stated; original panxu-ai.github.io redirects to panxulab.github.io</t>
         </is>
       </c>
       <c r="X55" t="inlineStr">
         <is>
-          <t>fit based on name-matched papers only: check they are this person's</t>
+          <t>dossier reader says A: Upgraded B-&gt;A: ML-core (RL, LLMs, data-efficient learning), tenure-track assistant professor with healthcare application</t>
         </is>
       </c>
     </row>
@@ -6014,12 +6026,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Wenpin Hou</t>
+          <t>Pixu Shi</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Assistant Professor in Biostatistics &amp; Bioinformatics</t>
+          <t>Assistant Professor of Biostatistics &amp; Bioinformatics</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -6039,47 +6051,35 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>AI-agent network structure compared with human social networks; scRNA dimensionality reduction.</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>multi-agent LLM systems</t>
-        </is>
-      </c>
+          <t>Trajectory-guided dimensionality reduction for multi-sample single-cell RNA-seq data.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>wenpin.hou@duke.edu</t>
+          <t>pixu.shi@duke.edu</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/profile/wenpin-hou</t>
+          <t>https://biostat.duke.edu/profile/pixu-shi</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>https://winnie09.github.io/Wenpin_Hou</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>MethylProphet: A Generalized Gene-Contextual Model for Inferring Whole-Genome DNA Methylation Landscape</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>Benchmarking large language models for genomic knowledge with GeneTuring</t>
-        </is>
-      </c>
+          <t>https://biostat.duke.edu/profile/pixu-shi</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Structural Divergence Between the Moltbook AI-Agent Network and Human Social Networks (2026) | Trajectory-guided dimensionality reduction for multi-sample single-cell RNA-seq data reveals biologically relevant sample-level heterogeneity (2026)</t>
+          <t>Branched chain amino acid metabolism and microbiome in adolescents with obesity during weight loss therapy (2026) | Characterizing the composition and diversity of the vaginal microbiome in ovarian cancer (2026)</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>https://biostat.duke.edu/people/faculty?page=2</t>
+          <t>https://biostat.duke.edu/people/faculty?page=5</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -6089,26 +6089,20 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>Yes: I have fundings to support 1-2 PhD students. If you are interested, please send me your CV and, at the same time, list me as your preferred mentor in your PhD application.</t>
-        </is>
-      </c>
-      <c r="T56" t="n">
-        <v>2026</v>
-      </c>
+          <t xml:space="preserve">Unspecified: </t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr"/>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>Her multimodal representation learning / foundation models for cells and 'one-shot learning and interpretability' paper connect to the applicant's BioCLIP-based fusion work and leakage-aware evaluation (arborphy).</t>
-        </is>
-      </c>
+      <c r="V56" t="inlineStr"/>
       <c r="W56" t="inlineStr">
         <is>
-          <t>start year 2026 inferred from Feb 2026 'Meet' article; Columbia appointment (research leave) still held; applicant is a Columbia student: lab collaborates with Columbia, mention nothing beyond applicant.yaml</t>
+          <t>no lab/personal site found (1 search); official profile has no research text; her 2026 Bioinformatics paper is listed only on Wenpin Hou's page, not hers, so not recorded as paper; recruiting info not found</t>
         </is>
       </c>
       <c r="X56" t="inlineStr">
         <is>
-          <t>fit based on name-matched papers only: check they are this person's; dossier reader says A: Upgraded B-&gt;A: Bio-AI foundation-model lab, new Duke assistant professor, explicitly funded for 1-2 PhD students and sta</t>
+          <t>fit based on name-matched papers only: check they are this person's</t>
         </is>
       </c>
     </row>
@@ -6118,27 +6112,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Icahn School of Medicine at Mount Sinai</t>
+          <t>Duke University</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Diagnostic, Molecular and Interventional Radiology</t>
+          <t>Biostatistics &amp; Bioinformatics (SOM); CBB program</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Christine Chen</t>
+          <t>Wenpin Hou</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ASSOCIATE PROFESSOR</t>
+          <t>Assistant Professor in Biostatistics &amp; Bioinformatics</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -6148,40 +6142,52 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>medical-AI</t>
+          <t>AI-for-science</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Radiology lab on ultrasound AI decision support for breast and sarcoma lesions; radiomics integration.</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr"/>
+          <t>AI-agent network structure compared with human social networks; scRNA dimensionality reduction.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>multi-agent LLM systems</t>
+        </is>
+      </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>christine.chen@mountsinai.org</t>
+          <t>wenpin.hou@duke.edu</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/christine-chen4</t>
+          <t>https://biostat.duke.edu/profile/wenpin-hou</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/christine-chen4</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr"/>
-      <c r="O57" t="inlineStr"/>
+          <t>https://winnie09.github.io/Wenpin_Hou</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>MethylProphet: A Generalized Gene-Contextual Model for Inferring Whole-Genome DNA Methylation Landscape</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Benchmarking large language models for genomic knowledge with GeneTuring</t>
+        </is>
+      </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Integration of advanced ultrasound techniques, radiomics, and artificial intelligence for improved diagnosis of cystic breast lesions (2026) | Breast lymphoma: Imaging features, clinical presentation, and ultrasound artificial intelligence (AI) decision support (DS) (2025)</t>
+          <t>Structural Divergence Between the Moltbook AI-Agent Network and Human Social Networks (2026) | Trajectory-guided dimensionality reduction for multi-sample single-cell RNA-seq data reveals biologically relevant sample-level heterogeneity (2026)</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=20</t>
+          <t>https://biostat.duke.edu/people/faculty?page=2</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -6191,20 +6197,26 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unspecified: </t>
-        </is>
-      </c>
-      <c r="T57" t="inlineStr"/>
+          <t>Yes: I have fundings to support 1-2 PhD students. If you are interested, please send me your CV and, at the same time, list me as your preferred mentor in your PhD application.</t>
+        </is>
+      </c>
+      <c r="T57" t="n">
+        <v>2026</v>
+      </c>
       <c r="U57" t="inlineStr"/>
-      <c r="V57" t="inlineStr"/>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Her multimodal representation learning / foundation models for cells and 'one-shot learning and interpretability' paper connect to the applicant's BioCLIP-based fusion work and leakage-aware evaluation (arborphy).</t>
+        </is>
+      </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>clinical radiologist (prostate MRI, TULSA lead); no lab site found on profile</t>
+          <t>start year 2026 inferred from Feb 2026 'Meet' article; Columbia appointment (research leave) still held; applicant is a Columbia student: lab collaborates with Columbia, mention nothing beyond applicant.yaml</t>
         </is>
       </c>
       <c r="X57" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile: Dr. Chen specializes in prostate MRI and MRI-guided interventions; clinical, no lab/ML group found (profile men</t>
+          <t>fit based on name-matched papers only: check they are this person's; dossier reader says A: Upgraded B-&gt;A: Bio-AI foundation-model lab, new Duke assistant professor, explicitly funded for 1-2 PhD students and sta</t>
         </is>
       </c>
     </row>
@@ -6219,22 +6231,22 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Genetics and Genomic Sciences</t>
+          <t>Diagnostic, Molecular and Interventional Radiology</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Erming Wang</t>
+          <t>Christine Chen</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ASSISTANT PROFESSOR</t>
+          <t>ASSOCIATE PROFESSOR</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -6244,40 +6256,40 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>AI-for-science</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Bioinformatics and systems-biology tools integrating omics data for Alzheimer disease.</t>
+          <t>Radiology lab on ultrasound AI decision support for breast and sarcoma lesions; radiomics integration.</t>
         </is>
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
-          <t>erming.wang@mssm.edu</t>
+          <t>christine.chen@mountsinai.org</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/erming-wang</t>
+          <t>https://profiles.icahn.mssm.edu/christine-chen4</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/erming-wang</t>
+          <t>https://profiles.icahn.mssm.edu/christine-chen4</t>
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Sex and APOE genotype specific brain regional vulnerability to Alzheimer's Disease (2026) | Molecular Networks and Key Regulators Underlying Resilience of the Human Brain to Aging and Dementia (2026)</t>
+          <t>Integration of advanced ultrasound techniques, radiomics, and artificial intelligence for improved diagnosis of cystic breast lesions (2026) | Breast lymphoma: Imaging features, clinical presentation, and ultrasound artificial intelligence (AI) decision support (DS) (2025)</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470001513038352&amp;selectedFilter=department&amp;tab=faculty&amp;start=120</t>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=20</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -6295,10 +6307,14 @@
       <c r="V58" t="inlineStr"/>
       <c r="W58" t="inlineStr">
         <is>
-          <t>no lab site found (2 searches); official profile only; no recruiting info</t>
-        </is>
-      </c>
-      <c r="X58" t="inlineStr"/>
+          <t>clinical radiologist (prostate MRI, TULSA lead); no lab site found on profile</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile: Dr. Chen specializes in prostate MRI and MRI-guided interventions; clinical, no lab/ML group found (profile men</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -6311,12 +6327,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Diagnostic, Molecular and Interventional Radiology; BMEII core + AI</t>
+          <t>Genetics and Genomic Sciences</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Hao Chih Lee</t>
+          <t>Erming Wang</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -6336,40 +6352,40 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>medical-AI</t>
+          <t>AI-for-science</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Cardiovascular imaging AI and deep learning; retinal imaging with supervised learning; LLM extraction from imaging reports.</t>
+          <t>Bioinformatics and systems-biology tools integrating omics data for Alzheimer disease.</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>hao-chih.lee@mssm.edu</t>
+          <t>erming.wang@mssm.edu</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/hao-chih-lee</t>
+          <t>https://profiles.icahn.mssm.edu/erming-wang</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/hao-chih-lee</t>
+          <t>https://profiles.icahn.mssm.edu/erming-wang</t>
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
         <is>
-          <t>AI and Deep Learning in Cardiovascular Imaging: From Risk Stratification to Precision Phenotyping (2026) | Retinal imaging and supervised learning predict hospitalizations and kidney and heart-lung damage in sickle cell disease (2026)</t>
+          <t>Sex and APOE genotype specific brain regional vulnerability to Alzheimer's Disease (2026) | Molecular Networks and Key Regulators Underlying Resilience of the Human Brain to Aging and Dementia (2026)</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=110</t>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470001513038352&amp;selectedFilter=department&amp;tab=faculty&amp;start=120</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -6387,14 +6403,10 @@
       <c r="V59" t="inlineStr"/>
       <c r="W59" t="inlineStr">
         <is>
-          <t>Radiology assistant prof; profile has no bio; no lab site found (WebSearch); co-founder of Crossmodal Intelligence Inc. per industry disclosure</t>
-        </is>
-      </c>
-      <c r="X59" t="inlineStr">
-        <is>
-          <t>fit based on name-matched papers only: check they are this person's; also listed as Hao-Chih Lee</t>
-        </is>
-      </c>
+          <t>no lab site found (2 searches); official profile only; no recruiting info</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -6407,22 +6419,22 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Diagnostic, Molecular and Interventional Radiology</t>
+          <t>Diagnostic, Molecular and Interventional Radiology; BMEII core + AI</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Michael S Chung</t>
+          <t>Hao Chih Lee</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ASSOCIATE PROFESSOR</t>
+          <t>ASSISTANT PROFESSOR</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -6437,35 +6449,35 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>NLP model predicting radiation pneumonitis; AI system integrating longitudinal data for lung disease.</t>
+          <t>Cardiovascular imaging AI and deep learning; retinal imaging with supervised learning; LLM extraction from imaging reports.</t>
         </is>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>michael.chung@mountsinai.org</t>
+          <t>hao-chih.lee@mssm.edu</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/michael-s-chung</t>
+          <t>https://profiles.icahn.mssm.edu/hao-chih-lee</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/michael-s-chung</t>
+          <t>https://profiles.icahn.mssm.edu/hao-chih-lee</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Natural language processing-based model to predict radiation pneumonitis in patients with locally advanced non-small cell lung cancer undergoing chemoradiotherapy: a retrospective cohort study (2026) | Postoperative CT surveillance in the evaluation of local recurrence after sub-lobar resection of neoplastic lesions of the lung (2024)</t>
+          <t>AI and Deep Learning in Cardiovascular Imaging: From Risk Stratification to Precision Phenotyping (2026) | Retinal imaging and supervised learning predict hospitalizations and kidney and heart-lung damage in sickle cell disease (2026)</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=30</t>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=110</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -6483,12 +6495,12 @@
       <c r="V60" t="inlineStr"/>
       <c r="W60" t="inlineStr">
         <is>
-          <t>clinical radiologist/cardiology; profile lists education only, no research or ML; no lab site</t>
+          <t>Radiology assistant prof; profile has no bio; no lab site found (WebSearch); co-founder of Crossmodal Intelligence Inc. per industry disclosure</t>
         </is>
       </c>
       <c r="X60" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile shows clinical radiology (cardiothoracic) credentials only; no ML research stated.</t>
+          <t>fit based on name-matched papers only: check they are this person's; also listed as Hao-Chih Lee</t>
         </is>
       </c>
     </row>
@@ -6508,7 +6520,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Mingqian Huang</t>
+          <t>Michael S Chung</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -6533,35 +6545,35 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Deep-learning knee MRI reconstruction; deepfake radiograph detection; DeepSeek LLM medical benchmarking.</t>
+          <t>NLP model predicting radiation pneumonitis; AI system integrating longitudinal data for lung disease.</t>
         </is>
       </c>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>mingqian.huang@mountsinai.org</t>
+          <t>michael.chung@mountsinai.org</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/mingqian-huang</t>
+          <t>https://profiles.icahn.mssm.edu/michael-s-chung</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/mingqian-huang</t>
+          <t>https://profiles.icahn.mssm.edu/michael-s-chung</t>
         </is>
       </c>
       <c r="N61" t="inlineStr"/>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
         <is>
-          <t>The Rise of Deepfake Medical Imaging: Radiologists' Diagnostic Accuracy in Detecting ChatGPT-generated Radiographs (2026) | Comparison of Deep-Learning-Based Reconstruction of Knee MRI with Conventional Sequences in Patients with Knee Pain (2026)</t>
+          <t>Natural language processing-based model to predict radiation pneumonitis in patients with locally advanced non-small cell lung cancer undergoing chemoradiotherapy: a retrospective cohort study (2026) | Postoperative CT surveillance in the evaluation of local recurrence after sub-lobar resection of neoplastic lesions of the lung (2024)</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=80</t>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=30</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
@@ -6579,12 +6591,12 @@
       <c r="V61" t="inlineStr"/>
       <c r="W61" t="inlineStr">
         <is>
-          <t>clinical MSK radiologist; profile lists education only, no research or ML; no lab site</t>
+          <t>clinical radiologist/cardiology; profile lists education only, no research or ML; no lab site</t>
         </is>
       </c>
       <c r="X61" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile shows clinical musculoskeletal radiology credentials only; no ML research stated.</t>
+          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile shows clinical radiology (cardiothoracic) credentials only; no ML research stated.</t>
         </is>
       </c>
     </row>
@@ -6599,12 +6611,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Genetics and Genomic Sciences</t>
+          <t>Diagnostic, Molecular and Interventional Radiology</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Won Min Song</t>
+          <t>Mingqian Huang</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -6624,44 +6636,40 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>AI-for-science</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Network modeling and embedding of multiscale proteomic and gene interaction data in Alzheimer disease.</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Bayesian SBM on connectome</t>
-        </is>
-      </c>
+          <t>Deep-learning knee MRI reconstruction; deepfake radiograph detection; DeepSeek LLM medical benchmarking.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>won-min.song@mssm.edu</t>
+          <t>mingqian.huang@mountsinai.org</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/won-min-song</t>
+          <t>https://profiles.icahn.mssm.edu/mingqian-huang</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>https://labs.icahn.mssm.edu/songlab/</t>
+          <t>https://profiles.icahn.mssm.edu/mingqian-huang</t>
         </is>
       </c>
       <c r="N62" t="inlineStr"/>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Multiscale proteomic modeling reveals protein networks driving Alzheimer's disease pathogenesis (2025) | DAP12 deletion reduces neuronal SLIT2 and demyelination and enhances brain resilience in female tauopathy mice (2025)</t>
+          <t>The Rise of Deepfake Medical Imaging: Radiologists' Diagnostic Accuracy in Detecting ChatGPT-generated Radiographs (2026) | Comparison of Deep-Learning-Based Reconstruction of Knee MRI with Conventional Sequences in Patients with Knee Pain (2026)</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470001513038352&amp;selectedFilter=department&amp;tab=faculty&amp;start=110</t>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470074622153001&amp;selectedFilter=department&amp;tab=faculty&amp;start=80</t>
         </is>
       </c>
       <c r="R62" t="inlineStr">
@@ -6671,28 +6679,20 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Unspecified: We are looking for another postdoc to join the lab.</t>
+          <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
       <c r="T62" t="inlineStr"/>
-      <c r="U62" t="inlineStr">
-        <is>
-          <t>Please send your CV, letter of intent, two recommendation letters to won-min.song@mssm.edu.</t>
-        </is>
-      </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>Network modeling for latent structure connects to the FlyWire Bayesian stochastic block model project.</t>
-        </is>
-      </c>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr"/>
       <c r="W62" t="inlineStr">
         <is>
-          <t>site looks stale (latest post Feb 2023; no paper after 2021 listed); hiring only a postdoc; start_year not found (associate)</t>
+          <t>clinical MSK radiologist; profile lists education only, no research or ML; no lab site</t>
         </is>
       </c>
       <c r="X62" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+</t>
+          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's; dossier reader says C: Profile shows clinical musculoskeletal radiology credentials only; no ML research stated.</t>
         </is>
       </c>
     </row>
@@ -6712,17 +6712,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Xianxiao Zhou</t>
+          <t>Won Min Song</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ASSISTANT PROFESSOR</t>
+          <t>ASSOCIATE PROFESSOR</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -6737,56 +6737,164 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Transcriptomic network models of neurodegenerative disease at single-cell level.</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr"/>
+          <t>Network modeling and embedding of multiscale proteomic and gene interaction data in Alzheimer disease.</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Bayesian SBM on connectome</t>
+        </is>
+      </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>xianxiao.zhou@mssm.edu</t>
+          <t>won-min.song@mssm.edu</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/xianxiao-zhou</t>
+          <t>https://profiles.icahn.mssm.edu/won-min-song</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>https://profiles.icahn.mssm.edu/xianxiao-zhou</t>
+          <t>https://labs.icahn.mssm.edu/songlab/</t>
         </is>
       </c>
       <c r="N63" t="inlineStr"/>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
         <is>
+          <t>Multiscale proteomic modeling reveals protein networks driving Alzheimer's disease pathogenesis (2025) | DAP12 deletion reduces neuronal SLIT2 and demyelination and enhances brain resilience in female tauopathy mice (2025)</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470001513038352&amp;selectedFilter=department&amp;tab=faculty&amp;start=110</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Unspecified: We are looking for another postdoc to join the lab.</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Please send your CV, letter of intent, two recommendation letters to won-min.song@mssm.edu.</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Network modeling for latent structure connects to the FlyWire Bayesian stochastic block model project.</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>site looks stale (latest post Feb 2023; no paper after 2021 listed); hiring only a postdoc; start_year not found (associate)</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>4</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Icahn School of Medicine at Mount Sinai</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Genetics and Genomic Sciences</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Xianxiao Zhou</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ASSISTANT PROFESSOR</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>AI-for-science</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Transcriptomic network models of neurodegenerative disease at single-cell level.</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>xianxiao.zhou@mssm.edu</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>https://profiles.icahn.mssm.edu/xianxiao-zhou</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>https://profiles.icahn.mssm.edu/xianxiao-zhou</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr">
+        <is>
           <t>Sex and APOE genotype specific brain regional vulnerability to Alzheimer's Disease (2026) | Multiscale Transcriptomic Network Models of Parkinson's Disease at the Single Cell Level (2026)</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q64" t="inlineStr">
         <is>
           <t>https://faculty.icahn.mssm.edu/results?departmentId=0000072470001513038352&amp;selectedFilter=department&amp;tab=faculty&amp;start=140</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
+      <c r="R64" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="S63" t="inlineStr">
+      <c r="S64" t="inlineStr">
         <is>
           <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
-      <c r="T63" t="inlineStr"/>
-      <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr">
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="inlineStr"/>
+      <c r="W64" t="inlineStr">
         <is>
           <t>profile has no bio; no lab site found (WebSearch x1)</t>
         </is>
       </c>
-      <c r="X63" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>fit based on name-matched papers only: check they are this person's</t>
         </is>
@@ -6803,7 +6911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X15"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7516,17 +7624,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Boston University</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Psychological &amp; Brain Sciences; Graduate Program for Neuroscience (faculty); Center for Systems Neuroscience</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Arthur Lee</t>
+          <t>Congyu Liao</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -7546,44 +7654,36 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Card has no research text or papers.</t>
+          <t>Developing diffusion and quantitative MRI techniques, magnetic resonance fingerprinting, for neurodevelopment.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>artlee@bu.edu</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>https://www.bu.edu/psych/profile/arthur-sangil-lee/</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>http://thedecodinglab.com/</t>
+          <t>https://researcherprofiles.org/profile/612476762</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Neural decoders: saving the baby from the bathwater</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Distinguishing deception from its confounds by improving the validity of fMRI-based neural prediction</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
+          <t>Effects of diffusion MRI spatial resolution on human brain short-range association fiber reconstruction and structural connectivity estimation (2026)</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Self-calibrated B&amp;lt;sub&amp;gt;1&amp;lt;/sub&amp;gt; &amp;lt;sup&amp;gt;+&amp;lt;/sup&amp;gt; and B&amp;lt;sub&amp;gt;0&amp;lt;/sub&amp;gt; Field Inhomogeneities Estimation (SAFE) in 3D Magnetic Resonance Fingerprinting (2026)</t>
+        </is>
+      </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>https://www.bu.edu/psych/people/faculty/</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -7593,30 +7693,20 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Yes: We are looking for Ph.D. students interested in our research.</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>Please feel free to send an email to Arthur (see contact) to let him know to look out for your application.</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>His interest in validating neural decoders (confounds, interpretability) connects to the EEG motor-imagery decoder with run-grouped validation.</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Unspecified: </t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>2025</v>
+      </c>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr">
         <is>
-          <t>psychology department; applications go through Psychology or Neuroscience program, not CS/Stats</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>also listed as Arthur Sangil Lee</t>
-        </is>
-      </c>
+          <t>no lab site found; radiology.ucsf.edu pages returned 403 (not bypassed); MRI physics/acquisition first; ML role unclear</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -7629,22 +7719,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Congyu Liao</t>
+          <t>Jian Shi</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7659,7 +7749,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Developing diffusion and quantitative MRI techniques, magnetic resonance fingerprinting, for neurodevelopment.</t>
+          <t>Machine learning with molecular experiments to decode Alzheimer disease, brain injury, brain tumor mechanisms.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -7667,23 +7757,19 @@
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/612476762</t>
+          <t>https://researcherprofiles.org/profile/681177372</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Effects of diffusion MRI spatial resolution on human brain short-range association fiber reconstruction and structural connectivity estimation (2026)</t>
+          <t>Blood Markers Show Neural Consequences of LongCOVID-19 (2024)</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Self-calibrated B&amp;lt;sub&amp;gt;1&amp;lt;/sub&amp;gt; &amp;lt;sup&amp;gt;+&amp;lt;/sup&amp;gt; and B&amp;lt;sub&amp;gt;0&amp;lt;/sub&amp;gt; Field Inhomogeneities Estimation (SAFE) in 3D Magnetic Resonance Fingerprinting (2026)</t>
-        </is>
-      </c>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -7696,17 +7782,19 @@
           <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
-      <c r="T9" t="n">
-        <v>2025</v>
-      </c>
+      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr">
         <is>
-          <t>no lab site found; radiology.ucsf.edu pages returned 403 (not bypassed); MRI physics/acquisition first; ML role unclear</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr"/>
+          <t>no lab site found; wet-lab neuroinflammation/stroke/glioblastoma group with ML as one tool; Associate Professor</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+; dossier reader says C: Biology-first (Alzheimer's, injury, tumors with animal models); ML is supporting.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -7719,22 +7807,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Jian Shi</t>
+          <t>Jonathan Liu</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -7749,7 +7837,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Machine learning with molecular experiments to decode Alzheimer disease, brain injury, brain tumor mechanisms.</t>
+          <t>Radiologist with quantitative SPECT methods and AI applications in thoracic and cardiovascular radiology.</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -7757,19 +7845,19 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/681177372</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>Blood Markers Show Neural Consequences of LongCOVID-19 (2024)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/319885321</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Multimodality Imaging in Myocarditis: Integrating Etiology, Diagnosis, and Risk Stratification (2026)</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -7782,17 +7870,19 @@
           <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>2022</v>
+      </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr">
         <is>
-          <t>no lab site found; wet-lab neuroinflammation/stroke/glioblastoma group with ML as one tool; Associate Professor</t>
+          <t>clinical thoracic radiologist; no lab; likely not a PhD advisor</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>associate: confirm promoted 2020+; dossier reader says C: Biology-first (Alzheimer's, injury, tumors with animal models); ML is supporting.</t>
+          <t>dossier reader says C: Clinical radiologist; AI is a side interest, no lab found.</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7902,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Jonathan Liu</t>
+          <t>Kang Wang</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -7837,22 +7927,30 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Radiologist with quantitative SPECT methods and AI applications in thoracic and cardiovascular radiology.</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>Develops anatomy-aware vision-language AI for CT detection of metastatic colorectal cancer.</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>BioCLIP/EfficientNet fusion (CV)</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/319885321</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/523574019</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Zero-Shot Large Language Model-Powered Data Curation for Pancreatic Cyst Surveillance: Promise, Progress, and the Path to Practice (2026)</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Multimodality Imaging in Myocarditis: Integrating Etiology, Diagnosis, and Risk Stratification (2026)</t>
+          <t>Imaging Evaluation for Steatotic Liver Disease (2026) | Diagnostic performance of CT/MRI LI-RADS radiation treatment response algorithm v2024 for Y-90 radioembolization (2026)</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -7870,21 +7968,15 @@
           <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
-      <c r="T11" t="n">
-        <v>2022</v>
-      </c>
+      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr">
         <is>
-          <t>clinical thoracic radiologist; no lab; likely not a PhD advisor</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>dossier reader says C: Clinical radiologist; AI is a side interest, no lab found.</t>
-        </is>
-      </c>
+          <t>no lab site; radiology.ucsf.edu 403 (not bypassed); web-search summary (not fetched page) says AI-based quantitative liver MRI, vision-language models for abdominal oncology, NIH R01 2025-2029</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -7902,7 +7994,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kang Wang</t>
+          <t>Maggie Chung</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -7927,32 +8019,28 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Develops anatomy-aware vision-language AI for CT detection of metastatic colorectal cancer.</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>BioCLIP/EfficientNet fusion (CV)</t>
-        </is>
-      </c>
+          <t>Breast imaging radiologist; deep learning synthetic contrast MRI, AI risk stratification, language-model report extraction.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/523574019</t>
+          <t>https://researcherprofiles.org/profile/14904495</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Zero-Shot Large Language Model-Powered Data Curation for Pancreatic Cyst Surveillance: Promise, Progress, and the Path to Practice (2026)</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Imaging Evaluation for Steatotic Liver Disease (2026) | Diagnostic performance of CT/MRI LI-RADS radiation treatment response algorithm v2024 for Y-90 radioembolization (2026)</t>
-        </is>
-      </c>
+          <t>Cryoablation Versus Breast-Conserving Surgery for Early-Stage, Low-Risk Breast Cancer ≤ 1.5 cm: A Cost-Effectiveness Analysis (2026)</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>From Risk Prediction to Coordinated Care (2026)</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr">
         <is>
           <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
@@ -7973,7 +8061,7 @@
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>no lab site; radiology.ucsf.edu 403 (not bypassed); web-search summary (not fetched page) says AI-based quantitative liver MRI, vision-language models for abdominal oncology, NIH R01 2025-2029</t>
+          <t>clinical breast radiologist (MD); no lab site found</t>
         </is>
       </c>
       <c r="X12" t="inlineStr"/>
@@ -7994,17 +8082,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Maggie Chung</t>
+          <t>Yan Li</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -8019,7 +8107,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Breast imaging radiologist; deep learning synthetic contrast MRI, AI risk stratification, language-model report extraction.</t>
+          <t>Brain MR spectroscopic imaging methods, statistical methods, and machine learning for glioma recurrence.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -8027,20 +8115,16 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/14904495</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>Cryoablation Versus Breast-Conserving Surgery for Early-Stage, Low-Risk Breast Cancer ≤ 1.5 cm: A Cost-Effectiveness Analysis (2026)</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>From Risk Prediction to Coordinated Care (2026)</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/189562</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Radiobiological dosimetry using hybrid imaging-derived spatiotemporal dose distributions for&amp;lt;sup&amp;gt;131&amp;lt;/sup&amp;gt;I therapy of metastatic thyroid cancer (2026) | Spatially identifying regions of tumor recurrence in patients with suspected recurrent glioma using physiologic MRI and machine learning (2026)</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
@@ -8061,10 +8145,14 @@
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>clinical breast radiologist (MD); no lab site found</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr"/>
+          <t>lab site lilabimaging.ucsf.edu returned 403 (not bypassed); no page text read; web search only: MR spectroscopic imaging methods, Associate Professor</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -8082,7 +8170,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Yan Li</t>
+          <t>Yang Yang</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -8107,7 +8195,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Brain MR spectroscopic imaging methods, statistical methods, and machine learning for glioma recurrence.</t>
+          <t>MRI sequence development, motion correction and AI; predicting Alzheimer outcomes from single MRI.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -8115,14 +8203,18 @@
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/189562</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/327403539</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Predicting categorical and continuous Alzheimer's disease outcomes from a single MRI scan (2026)</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Radiobiological dosimetry using hybrid imaging-derived spatiotemporal dose distributions for&amp;lt;sup&amp;gt;131&amp;lt;/sup&amp;gt;I therapy of metastatic thyroid cancer (2026) | Spatially identifying regions of tumor recurrence in patients with suspected recurrent glioma using physiologic MRI and machine learning (2026)</t>
+          <t>Determinants of image quality in respiratory triggered free breathing lung MRI at 0.55 T in adults (2026) | Self-calibrated B&amp;lt;sub&amp;gt;1&amp;lt;/sub&amp;gt; &amp;lt;sup&amp;gt;+&amp;lt;/sup&amp;gt; and B&amp;lt;sub&amp;gt;0&amp;lt;/sub&amp;gt; Field Inhomogeneities Estimation (SAFE) in 3D Magnetic Resonance Fingerprinting (2026)</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -8145,102 +8237,10 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr">
         <is>
-          <t>lab site lilabimaging.ucsf.edu returned 403 (not bypassed); no page text read; web search only: MR spectroscopic imaging methods, Associate Professor</t>
+          <t>no lab site found; MR sequence/physics first; AI component per search summary only</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>University of California San Francisco</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Radiology and Biomedical Imaging</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Yang Yang</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Associate Professor</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>associate</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>medical-AI</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>MRI sequence development, motion correction and AI; predicting Alzheimer outcomes from single MRI.</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>https://researcherprofiles.org/profile/327403539</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Predicting categorical and continuous Alzheimer's disease outcomes from a single MRI scan (2026)</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>Determinants of image quality in respiratory triggered free breathing lung MRI at 0.55 T in adults (2026) | Self-calibrated B&amp;lt;sub&amp;gt;1&amp;lt;/sub&amp;gt; &amp;lt;sup&amp;gt;+&amp;lt;/sup&amp;gt; and B&amp;lt;sub&amp;gt;0&amp;lt;/sub&amp;gt; Field Inhomogeneities Estimation (SAFE) in 3D Magnetic Resonance Fingerprinting (2026)</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="S15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unspecified: </t>
-        </is>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>no lab site found; MR sequence/physics first; AI component per search summary only</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
         <is>
           <t>associate: confirm promoted 2020+</t>
         </is>
@@ -24663,7 +24663,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>people 10 | need email 2 | check 1 | dropped C 18</t>
+          <t>people 11 | need email 1 | check 1 | dropped C 18</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>

</xml_diff>

<commit_message>
UCSF Neuroscience faculty from applicant-saved page (99, parsed by code); UC titles: Asst/Assoc abbreviations and 'in Residence' series now count as PhD-advising (+test); 4 new people tagged C
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHXVUB5nxWZdDwRJd5MuyH
</commit_message>
<xml_diff>
--- a/data/export/batch1.xlsx
+++ b/data/export/batch1.xlsx
@@ -12211,7 +12211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X153"/>
+  <dimension ref="A1:X157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Biological and Medical Informatics (BMI) PhD program core+affiliate faculty (Wayback 2026-05 copy); Neurology</t>
+          <t>Biological and Medical Informatics (BMI) PhD program core+affiliate faculty (Wayback 2026-05 copy); Neurology; Neuroscience Graduate Program (faculty)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -20705,17 +20705,17 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Cell and Tissue Biology</t>
+          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Bo Gong</t>
+          <t>Benjamin Huang</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Asst Professor in Residence</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -20735,7 +20735,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Cell biology of cell fate decisions in development and neurodegeneration.</t>
+          <t>Pediatric leukemia biology and clinical outcomes (MD, Pediatrics-Oncology)</t>
         </is>
       </c>
       <c r="J106" t="inlineStr"/>
@@ -20743,23 +20743,19 @@
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/686563008</t>
-        </is>
-      </c>
-      <c r="N106" t="inlineStr">
-        <is>
-          <t>Pulling the Back to Steer Cell Migration: Mechanisms of Structural Polarity in Confining Signaling and Protrusion (2026)</t>
-        </is>
-      </c>
+          <t>https://bms.ucsf.edu/people/benjamin-huang-md</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr"/>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
         <is>
-          <t>SEC14L2 couples chaperone-mediated autophagy to microtubule stability by targeting Stathmin 1 (2026)</t>
+          <t>Multiselective RAS(ON) inhibition targets oncogenic RAS and overcomes RAS-mediated resistance to FLT3i and BCL2i in AML (2026) | Reactive oxygen species define leukemia stem cell identity in pediatric acute myeloid leukemia (2026)</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Cell and Tissue Biology)</t>
+          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=10</t>
         </is>
       </c>
       <c r="R106" t="inlineStr"/>
@@ -20781,12 +20777,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Cell and Tissue Biology</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Bo Hu</t>
+          <t>Bo Gong</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -20811,7 +20807,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Intravenous ketamine protocol for psychiatric conditions in medical and surgical units.</t>
+          <t>Cell biology of cell fate decisions in development and neurodegeneration.</t>
         </is>
       </c>
       <c r="J107" t="inlineStr"/>
@@ -20819,19 +20815,23 @@
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/518025861</t>
+          <t>https://researcherprofiles.org/profile/686563008</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>Implementation and Preliminary Evaluation of an Intravenous Ketamine Protocol for Psychiatric Conditions in Medical and Surgical Units: A 1-Year Pilot Study (2026)</t>
+          <t>Pulling the Back to Steer Cell Migration: Mechanisms of Structural Polarity in Confining Signaling and Protrusion (2026)</t>
         </is>
       </c>
       <c r="O107" t="inlineStr"/>
-      <c r="P107" t="inlineStr"/>
+      <c r="P107" t="inlineStr">
+        <is>
+          <t>SEC14L2 couples chaperone-mediated autophagy to microtubule stability by targeting Stathmin 1 (2026)</t>
+        </is>
+      </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Cell and Tissue Biology)</t>
         </is>
       </c>
       <c r="R107" t="inlineStr"/>
@@ -20853,16 +20853,24 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Quantitative Biosciences Institute (home dept: Pharmaceutical Chemistry)</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Bo Huang</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
+          <t>Bo Hu</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr">
         <is>
           <t>C</t>
@@ -20875,7 +20883,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Fluorescence microscopy binders and transcriptional condensates.</t>
+          <t>Intravenous ketamine protocol for psychiatric conditions in medical and surgical units.</t>
         </is>
       </c>
       <c r="J108" t="inlineStr"/>
@@ -20883,19 +20891,19 @@
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
-          <t>http://huanglab.ucsf.edu</t>
-        </is>
-      </c>
-      <c r="N108" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/518025861</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Implementation and Preliminary Evaluation of an Intravenous Ketamine Protocol for Psychiatric Conditions in Medical and Surgical Units: A 1-Year Pilot Study (2026)</t>
+        </is>
+      </c>
       <c r="O108" t="inlineStr"/>
-      <c r="P108" t="inlineStr">
-        <is>
-          <t>De novo pan-rhodamine binders for fluorescence microscopy from mammalian cells to extremophiles (2026) | YAP charge patterning mediates signal integration through transcriptional co-condensates (2025)</t>
-        </is>
-      </c>
+      <c r="P108" t="inlineStr"/>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>https://qbi.ucsf.edu/investigators</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
         </is>
       </c>
       <c r="R108" t="inlineStr"/>
@@ -20917,24 +20925,16 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Quantitative Biosciences Institute (home dept: Pharmaceutical Chemistry)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Charlie Wang</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Assistant Professor</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
+          <t>Bo Huang</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>C</t>
@@ -20947,7 +20947,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Hyperpolarized 13C MRI for brain perfusion and glioma; imaging physics without ML.</t>
+          <t>Fluorescence microscopy binders and transcriptional condensates.</t>
         </is>
       </c>
       <c r="J109" t="inlineStr"/>
@@ -20955,27 +20955,19 @@
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/126038969</t>
-        </is>
-      </c>
-      <c r="N109" t="inlineStr">
-        <is>
-          <t>Translation of hyperpolarized [13C,15N2]urea MRI for novel human brain perfusion studies (2025)</t>
-        </is>
-      </c>
-      <c r="O109" t="inlineStr">
-        <is>
-          <t>A flexible MRF approach to improve kinetic rate estimation with bSSFP‐based hyperpolarized [1‐ 13C]pyruvate MRI (2025)</t>
-        </is>
-      </c>
+          <t>http://huanglab.ucsf.edu</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr">
         <is>
-          <t>IMG-97. Advancing hyperpolarized13C MRI for non-invasive assessment of blood-brain barrier integrity and IDH mutation status in glioma (2025)</t>
+          <t>De novo pan-rhodamine binders for fluorescence microscopy from mammalian cells to extremophiles (2026) | YAP charge patterning mediates signal integration through transcriptional co-condensates (2025)</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://qbi.ucsf.edu/investigators</t>
         </is>
       </c>
       <c r="R109" t="inlineStr"/>
@@ -21002,7 +20994,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Cheng Hong</t>
+          <t>Charlie Wang</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -21027,7 +21019,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Clinical liver MRI and LI-RADS imaging evaluation studies.</t>
+          <t>Hyperpolarized 13C MRI for brain perfusion and glioma; imaging physics without ML.</t>
         </is>
       </c>
       <c r="J110" t="inlineStr"/>
@@ -21035,22 +21027,22 @@
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/328148685</t>
+          <t>https://researcherprofiles.org/profile/126038969</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>Imaging Evaluation for Steatotic Liver Disease (2026)</t>
+          <t>Translation of hyperpolarized [13C,15N2]urea MRI for novel human brain perfusion studies (2025)</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>Diagnostic performance of CT/MRI LI-RADS radiation treatment response algorithm v2024 for Y-90 radioembolization (2026)</t>
+          <t>A flexible MRF approach to improve kinetic rate estimation with bSSFP‐based hyperpolarized [1‐ 13C]pyruvate MRI (2025)</t>
         </is>
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>Lessons learned: strategies for implementing and the ongoing use of LI-RADS in your practice (2025)</t>
+          <t>IMG-97. Advancing hyperpolarized13C MRI for non-invasive assessment of blood-brain barrier integrity and IDH mutation status in glioma (2025)</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -21077,12 +21069,12 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Cheng Qian</t>
+          <t>Cheng Hong</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -21107,7 +21099,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Psychiatry; child behavioral health programs, clinical training lead.</t>
+          <t>Clinical liver MRI and LI-RADS imaging evaluation studies.</t>
         </is>
       </c>
       <c r="J111" t="inlineStr"/>
@@ -21115,15 +21107,27 @@
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/343574317</t>
-        </is>
-      </c>
-      <c r="N111" t="inlineStr"/>
-      <c r="O111" t="inlineStr"/>
-      <c r="P111" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/328148685</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Imaging Evaluation for Steatotic Liver Disease (2026)</t>
+        </is>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Diagnostic performance of CT/MRI LI-RADS radiation treatment response algorithm v2024 for Y-90 radioembolization (2026)</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>Lessons learned: strategies for implementing and the ongoing use of LI-RADS in your practice (2025)</t>
+        </is>
+      </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R111" t="inlineStr"/>
@@ -21150,17 +21154,17 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Chuan Mei Lee</t>
+          <t>Cheng Qian</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -21175,7 +21179,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Child psychiatry access programs and integration of mental health services in pediatric primary care.</t>
+          <t>Psychiatry; child behavioral health programs, clinical training lead.</t>
         </is>
       </c>
       <c r="J112" t="inlineStr"/>
@@ -21183,24 +21187,12 @@
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/188250</t>
-        </is>
-      </c>
-      <c r="N112" t="inlineStr">
-        <is>
-          <t>Location of Crisis Service Delivery for Medicaid-Enrolled Youths with Behavioral Health Conditions (2026)</t>
-        </is>
-      </c>
-      <c r="O112" t="inlineStr">
-        <is>
-          <t>Substance Use Services at Child Psychiatry Access Programs. (2026)</t>
-        </is>
-      </c>
-      <c r="P112" t="inlineStr">
-        <is>
-          <t>5.24 Behavioral Problems and Chronic Pain Among Children and Adolescents in the United States: An Analysis From 2016 to 2023 (2025) | 4.74 Addressing the Youth Mental Health Crisis Through Psychiatric Consultation to Primary Care: The California Child and Adolescent Mental Health Access Program (2025)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/343574317</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
+      <c r="P112" t="inlineStr"/>
       <c r="Q112" t="inlineStr">
         <is>
           <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
@@ -21212,11 +21204,7 @@
       <c r="U112" t="inlineStr"/>
       <c r="V112" t="inlineStr"/>
       <c r="W112" t="inlineStr"/>
-      <c r="X112" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -21229,22 +21217,22 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Connie Lu</t>
+          <t>Chuan Mei Lee</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -21259,7 +21247,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Radiology MD; diagnostic radiology residency, clinical profile.</t>
+          <t>Child psychiatry access programs and integration of mental health services in pediatric primary care.</t>
         </is>
       </c>
       <c r="J113" t="inlineStr"/>
@@ -21267,15 +21255,27 @@
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/681177355</t>
-        </is>
-      </c>
-      <c r="N113" t="inlineStr"/>
-      <c r="O113" t="inlineStr"/>
-      <c r="P113" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/188250</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>Location of Crisis Service Delivery for Medicaid-Enrolled Youths with Behavioral Health Conditions (2026)</t>
+        </is>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Substance Use Services at Child Psychiatry Access Programs. (2026)</t>
+        </is>
+      </c>
+      <c r="P113" t="inlineStr">
+        <is>
+          <t>5.24 Behavioral Problems and Chronic Pain Among Children and Adolescents in the United States: An Analysis From 2016 to 2023 (2025) | 4.74 Addressing the Youth Mental Health Crisis Through Psychiatric Consultation to Primary Care: The California Child and Adolescent Mental Health Access Program (2025)</t>
+        </is>
+      </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
         </is>
       </c>
       <c r="R113" t="inlineStr"/>
@@ -21284,7 +21284,11 @@
       <c r="U113" t="inlineStr"/>
       <c r="V113" t="inlineStr"/>
       <c r="W113" t="inlineStr"/>
-      <c r="X113" t="inlineStr"/>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -21297,12 +21301,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only)</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Edward Hsiao</t>
+          <t>Connie Lu</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -21327,7 +21331,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Patient-reported outcomes and trials for fibrodysplasia ossificans progressiva and fibrous dysplasia.</t>
+          <t>Radiology MD; diagnostic radiology residency, clinical profile.</t>
         </is>
       </c>
       <c r="J114" t="inlineStr"/>
@@ -21335,19 +21339,15 @@
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
-          <t>https://bms.ucsf.edu/people/edward-hsiao-md-phd</t>
+          <t>https://researcherprofiles.org/profile/681177355</t>
         </is>
       </c>
       <c r="N114" t="inlineStr"/>
       <c r="O114" t="inlineStr"/>
-      <c r="P114" t="inlineStr">
-        <is>
-          <t>Development of the Fibrodysplasia Ossificans Progressiva FLare EXperience Revised (FOP-FLEX-R©) Questionnaire: A Patient-Reported Outcome Measure (2026) | Palovarotene impact on fibrodysplasia ossificans progressiva (FOP): data from month 48 of the phase III MOVE trial (2026)</t>
-        </is>
-      </c>
+      <c r="P114" t="inlineStr"/>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=10</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R114" t="inlineStr"/>
@@ -21369,22 +21369,22 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only)</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Ellen Chang</t>
+          <t>Edward Hsiao</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -21399,7 +21399,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Nasopharyngeal carcinoma screening and population survival epidemiology.</t>
+          <t>Patient-reported outcomes and trials for fibrodysplasia ossificans progressiva and fibrous dysplasia.</t>
         </is>
       </c>
       <c r="J115" t="inlineStr"/>
@@ -21407,19 +21407,19 @@
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/327403537</t>
-        </is>
-      </c>
-      <c r="N115" t="inlineStr">
-        <is>
-          <t>Population-based nasopharyngeal carcinoma survival in southern China (2026)</t>
-        </is>
-      </c>
+          <t>https://bms.ucsf.edu/people/edward-hsiao-md-phd</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr"/>
       <c r="O115" t="inlineStr"/>
-      <c r="P115" t="inlineStr"/>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>Development of the Fibrodysplasia Ossificans Progressiva FLare EXperience Revised (FOP-FLEX-R©) Questionnaire: A Patient-Reported Outcome Measure (2026) | Palovarotene impact on fibrodysplasia ossificans progressiva (FOP): data from month 48 of the phase III MOVE trial (2026)</t>
+        </is>
+      </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=10</t>
         </is>
       </c>
       <c r="R115" t="inlineStr"/>
@@ -21428,11 +21428,7 @@
       <c r="U115" t="inlineStr"/>
       <c r="V115" t="inlineStr"/>
       <c r="W115" t="inlineStr"/>
-      <c r="X115" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -21445,12 +21441,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Biochemistry and Biophysics</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Eric Chow</t>
+          <t>Ellen Chang</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -21475,7 +21471,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Single-cell multiomic CRISPR screens and compact guide RNA libraries for gene regulation.</t>
+          <t>Nasopharyngeal carcinoma screening and population survival epidemiology.</t>
         </is>
       </c>
       <c r="J116" t="inlineStr"/>
@@ -21483,23 +21479,19 @@
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/185237</t>
+          <t>https://researcherprofiles.org/profile/327403537</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>Simultaneous capture of single cell RNA-seq, ATAC-seq, and CRISPR perturbation enables multiomic screens to identify gene regulatory relationships (2025)</t>
-        </is>
-      </c>
-      <c r="O116" t="inlineStr">
-        <is>
-          <t>Compact CRISPR genetic screens enabled by improved guide RNA library cloning (2024)</t>
-        </is>
-      </c>
+          <t>Population-based nasopharyngeal carcinoma survival in southern China (2026)</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr"/>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Biochemistry and Biophysics)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R116" t="inlineStr"/>
@@ -21525,22 +21517,22 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Biochemistry and Biophysics</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Greta Peng</t>
+          <t>Eric Chow</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -21555,7 +21547,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Neurohumanities education and neurology outcomes in neonatal seizures and DIPG.</t>
+          <t>Single-cell multiomic CRISPR screens and compact guide RNA libraries for gene regulation.</t>
         </is>
       </c>
       <c r="J117" t="inlineStr"/>
@@ -21563,23 +21555,23 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/308694444</t>
+          <t>https://researcherprofiles.org/profile/185237</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>The DIPG/DMG National Tumor Board: The power of advocacy (2026)</t>
+          <t>Simultaneous capture of single cell RNA-seq, ATAC-seq, and CRISPR perturbation enables multiomic screens to identify gene regulatory relationships (2025)</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Preferred Parental Language and Neurodevelopmental Outcomes Among Infants With Acute Provoked Neonatal Seizures in the United States (2025)</t>
+          <t>Compact CRISPR genetic screens enabled by improved guide RNA library cloning (2024)</t>
         </is>
       </c>
       <c r="P117" t="inlineStr"/>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Biochemistry and Biophysics)</t>
         </is>
       </c>
       <c r="R117" t="inlineStr"/>
@@ -21588,7 +21580,11 @@
       <c r="U117" t="inlineStr"/>
       <c r="V117" t="inlineStr"/>
       <c r="W117" t="inlineStr"/>
-      <c r="X117" t="inlineStr"/>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -21601,16 +21597,24 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Quantitative Biosciences Institute (home dept: Biochemistry &amp; Biophysics)</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Hao Li</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
+          <t>Greta Peng</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
       <c r="G118" t="inlineStr">
         <is>
           <t>C</t>
@@ -21623,7 +21627,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Molecular mechanisms of aging, genetic determinants of complex traits, gene regulatory networks.</t>
+          <t>Neurohumanities education and neurology outcomes in neonatal seizures and DIPG.</t>
         </is>
       </c>
       <c r="J118" t="inlineStr"/>
@@ -21631,19 +21635,23 @@
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
-          <t>http://mobydick.ucsf.edu/</t>
-        </is>
-      </c>
-      <c r="N118" t="inlineStr"/>
-      <c r="O118" t="inlineStr"/>
-      <c r="P118" t="inlineStr">
-        <is>
-          <t>Inferring Gene Regulatory Network Architecture Underlying Complex Traits: An Integrative Analysis of Mutant Lifespan and Gene Expression Profiles Identifies Master Regulators and Key Functional Modules for Yeast Aging (2026) | Complement C4b as a key mediator of synaptic loss and cognitive decline in brain aging (2025)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/308694444</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>The DIPG/DMG National Tumor Board: The power of advocacy (2026)</t>
+        </is>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Preferred Parental Language and Neurodevelopmental Outcomes Among Infants With Acute Provoked Neonatal Seizures in the United States (2025)</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr"/>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>https://qbi.ucsf.edu/investigators</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R118" t="inlineStr"/>
@@ -21665,24 +21673,16 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Quantitative Biosciences Institute (home dept: Biochemistry &amp; Biophysics)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Hohui Wang</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Associate Professor</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>associate</t>
-        </is>
-      </c>
+          <t>Hao Li</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>C</t>
@@ -21695,7 +21695,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Inflammatory bowel disease links to depression, dementia and suicide risk.</t>
+          <t>Molecular mechanisms of aging, genetic determinants of complex traits, gene regulatory networks.</t>
         </is>
       </c>
       <c r="J119" t="inlineStr"/>
@@ -21703,23 +21703,19 @@
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/195581</t>
-        </is>
-      </c>
-      <c r="N119" t="inlineStr">
-        <is>
-          <t>Inflammatory Bowel Disease and Neurodegenerative Diseases (2023)</t>
-        </is>
-      </c>
-      <c r="O119" t="inlineStr">
-        <is>
-          <t>Risk of Attempted Suicide Among Patients With IBD: A Nationwide Longitudinal Follow-up Study (2023)</t>
-        </is>
-      </c>
-      <c r="P119" t="inlineStr"/>
+          <t>http://mobydick.ucsf.edu/</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>Inferring Gene Regulatory Network Architecture Underlying Complex Traits: An Integrative Analysis of Mutant Lifespan and Gene Expression Profiles Identifies Master Regulators and Key Functional Modules for Yeast Aging (2026) | Complement C4b as a key mediator of synaptic loss and cognitive decline in brain aging (2025)</t>
+        </is>
+      </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
+          <t>https://qbi.ucsf.edu/investigators</t>
         </is>
       </c>
       <c r="R119" t="inlineStr"/>
@@ -21728,11 +21724,7 @@
       <c r="U119" t="inlineStr"/>
       <c r="V119" t="inlineStr"/>
       <c r="W119" t="inlineStr"/>
-      <c r="X119" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -21750,17 +21742,17 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Jessica Hua</t>
+          <t>Hohui Wang</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -21775,7 +21767,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Neuromodulation and cognition in schizophrenia; cortical thickness and social determinants.</t>
+          <t>Inflammatory bowel disease links to depression, dementia and suicide risk.</t>
         </is>
       </c>
       <c r="J120" t="inlineStr"/>
@@ -21783,17 +21775,17 @@
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/371173157</t>
+          <t>https://researcherprofiles.org/profile/195581</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>Social Determinants of Health and Neurobiology Across the Schizophrenia Course: A Systematic Review (2026)</t>
+          <t>Inflammatory Bowel Disease and Neurodegenerative Diseases (2023)</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Adjustment of Regional Cortical Thickness Measures for Global Cortical Thickness Obscures Deficits Across the Schizophrenia Spectrum: A Cautionary Note About Normative Modeling of Brain Imaging Data (2025)</t>
+          <t>Risk of Attempted Suicide Among Patients With IBD: A Nationwide Longitudinal Follow-up Study (2023)</t>
         </is>
       </c>
       <c r="P120" t="inlineStr"/>
@@ -21808,7 +21800,11 @@
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="inlineStr"/>
       <c r="W120" t="inlineStr"/>
-      <c r="X120" t="inlineStr"/>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -21821,12 +21817,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Neurological Surgery</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>John Yue</t>
+          <t>Jessica Hua</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -21851,7 +21847,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Blood-based biomarkers for brain injury classification and prognosis.</t>
+          <t>Neuromodulation and cognition in schizophrenia; cortical thickness and social determinants.</t>
         </is>
       </c>
       <c r="J121" t="inlineStr"/>
@@ -21859,23 +21855,23 @@
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/176762</t>
+          <t>https://researcherprofiles.org/profile/371173157</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>Clinical Utility of Structural Blood-Based Biomarkers in Pediatric Traumatic Brain Injury: A Focused Review of Glial Fibrillary Acidic Protein, Ubiquitin C-Terminal Hydrolase L1, and S100 Calcium-Binding Protein B (2026)</t>
+          <t>Social Determinants of Health and Neurobiology Across the Schizophrenia Course: A Systematic Review (2026)</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>Insurance-based disparities in traumatic brain injury length of stay and discharge dispositions: A retrospective cohort analysis of the national trauma data bank (2026)</t>
+          <t>Adjustment of Regional Cortical Thickness Measures for Global Cortical Thickness Obscures Deficits Across the Schizophrenia Spectrum: A Cautionary Note About Normative Modeling of Brain Imaging Data (2025)</t>
         </is>
       </c>
       <c r="P121" t="inlineStr"/>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
         </is>
       </c>
       <c r="R121" t="inlineStr"/>
@@ -21897,16 +21893,24 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Quantitative Biosciences Institute (home dept: Bioengineering)</t>
+          <t>Neurological Surgery</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Kevin Lou</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
+          <t>John Yue</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
       <c r="G122" t="inlineStr">
         <is>
           <t>C</t>
@@ -21919,7 +21923,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Kinase inhibitor design; clinical trial listing in neuro-oncology.</t>
+          <t>Blood-based biomarkers for brain injury classification and prognosis.</t>
         </is>
       </c>
       <c r="J122" t="inlineStr"/>
@@ -21927,19 +21931,23 @@
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/kevin.lou</t>
+          <t>https://researcherprofiles.org/profile/176762</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>A design approach for bitopic kinase inhibitors (2026)</t>
-        </is>
-      </c>
-      <c r="O122" t="inlineStr"/>
+          <t>Clinical Utility of Structural Blood-Based Biomarkers in Pediatric Traumatic Brain Injury: A Focused Review of Glial Fibrillary Acidic Protein, Ubiquitin C-Terminal Hydrolase L1, and S100 Calcium-Binding Protein B (2026)</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Insurance-based disparities in traumatic brain injury length of stay and discharge dispositions: A retrospective cohort analysis of the national trauma data bank (2026)</t>
+        </is>
+      </c>
       <c r="P122" t="inlineStr"/>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>https://qbi.ucsf.edu/investigators</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
         </is>
       </c>
       <c r="R122" t="inlineStr"/>
@@ -21961,22 +21969,22 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Neurological Surgery</t>
+          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only)</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Lee Tan</t>
+          <t>Jonathan Chou</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Asst. Professor In Residence</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -21991,7 +21999,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Minimally invasive and open spine surgery, including robotic and motion-preservation techniques.</t>
+          <t>Cancer cell biology and clinical oncology trials (MD/PhD, Hematology-Oncology)</t>
         </is>
       </c>
       <c r="J123" t="inlineStr"/>
@@ -21999,27 +22007,19 @@
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/196680</t>
-        </is>
-      </c>
-      <c r="N123" t="inlineStr">
-        <is>
-          <t>When Is Fusion Necessary in Addressing Symptomatic Adjacent Level Pathology - A Commentary on "How to Treat Adjacent-Segment Pathology Following Lumbar Fusion Surgery: Decompression Alone or Decompression With Extended Fusion Surgery?" (2026)</t>
-        </is>
-      </c>
-      <c r="O123" t="inlineStr">
-        <is>
-          <t>Safety and Efficacy of Real-Time Intraoperative Ultrasound-Guided Posterolateral Thoracic Diskectomy: Using Technology to Minimize Complication and Improve Surgical Outcome (2026)</t>
-        </is>
-      </c>
+          <t>https://bms.ucsf.edu/people/jonathan-chou-md-phd</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
         <is>
-          <t>Risk Factors, Biomechanics, and Prevention Strategies for Proximal Junctional Failure in Adult Spinal Deformity Surgery - A Commentary on "Proximal Junctional Failure Development Despite Achieving Ideal Sagittal Correction According to Age-Adjusted Alignment Target in Patients With Adult Spinal Deformity: Risk Factor Analysis of 196 Cases Undergoing Low Thoracic to Pelvic Fusion" (2024)</t>
+          <t>Autophagolysosomal exocytosis inverts Src kinase onto the cell surface in cancer (2026) | Prognostic Implications of Personalized Circulating Tumor DNA Testing in Patients with Advanced Urothelial Carcinoma Treated with Enfortumab Vedotin ± Pembrolizumab (2026)</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
+          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=5</t>
         </is>
       </c>
       <c r="R123" t="inlineStr"/>
@@ -22028,11 +22028,7 @@
       <c r="U123" t="inlineStr"/>
       <c r="V123" t="inlineStr"/>
       <c r="W123" t="inlineStr"/>
-      <c r="X123" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -22045,24 +22041,16 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Quantitative Biosciences Institute (home dept: Bioengineering)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Ling-Ya Chao</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Assistant Professor</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
+          <t>Kevin Lou</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>C</t>
@@ -22075,7 +22063,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Meta-analysis of bilateral centromedian nucleus neuromodulation for epilepsy.</t>
+          <t>Kinase inhibitor design; clinical trial listing in neuro-oncology.</t>
         </is>
       </c>
       <c r="J124" t="inlineStr"/>
@@ -22083,19 +22071,19 @@
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/695092660</t>
+          <t>https://profiles.ucsf.edu/kevin.lou</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>Systematic Review and Meta-Analysis of Bilateral Centromedian Nucleus Neuromodulation for Multifocal and Generalized Epilepsy. (2025)</t>
+          <t>A design approach for bitopic kinase inhibitors (2026)</t>
         </is>
       </c>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr"/>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://qbi.ucsf.edu/investigators</t>
         </is>
       </c>
       <c r="R124" t="inlineStr"/>
@@ -22117,12 +22105,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Neurological Surgery</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Min Kang</t>
+          <t>Lee Tan</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -22147,7 +22135,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Multidisciplinary care and clinical trials in myasthenia gravis.</t>
+          <t>Minimally invasive and open spine surgery, including robotic and motion-preservation techniques.</t>
         </is>
       </c>
       <c r="J125" t="inlineStr"/>
@@ -22155,19 +22143,27 @@
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/181165</t>
-        </is>
-      </c>
-      <c r="N125" t="inlineStr"/>
-      <c r="O125" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/196680</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>When Is Fusion Necessary in Addressing Symptomatic Adjacent Level Pathology - A Commentary on "How to Treat Adjacent-Segment Pathology Following Lumbar Fusion Surgery: Decompression Alone or Decompression With Extended Fusion Surgery?" (2026)</t>
+        </is>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Safety and Efficacy of Real-Time Intraoperative Ultrasound-Guided Posterolateral Thoracic Diskectomy: Using Technology to Minimize Complication and Improve Surgical Outcome (2026)</t>
+        </is>
+      </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>Optimising well-being in myasthenia gravis: a multidisciplinary approach (2026) | Switching to subcutaneous zilucoplan from intravenous complement component 5 inhibitors in generalised myasthenia gravis: a phase IIIb, open-label study (2025)</t>
+          <t>Risk Factors, Biomechanics, and Prevention Strategies for Proximal Junctional Failure in Adult Spinal Deformity Surgery - A Commentary on "Proximal Junctional Failure Development Despite Achieving Ideal Sagittal Correction According to Age-Adjusted Alignment Target in Patients With Adult Spinal Deformity: Risk Factor Analysis of 196 Cases Undergoing Low Thoracic to Pelvic Fusion" (2024)</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
         </is>
       </c>
       <c r="R125" t="inlineStr"/>
@@ -22193,12 +22189,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Neurological Surgery</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Ritchie Chen</t>
+          <t>Ling-Ya Chao</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -22223,7 +22219,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Engineers genetically targeted bioelectronic and optogenetic tools to map and control brain-body circuits.</t>
+          <t>Meta-analysis of bilateral centromedian nucleus neuromodulation for epilepsy.</t>
         </is>
       </c>
       <c r="J126" t="inlineStr"/>
@@ -22231,23 +22227,19 @@
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/359584750</t>
+          <t>https://researcherprofiles.org/profile/695092660</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>Interoceptive modulation of emotions (2025)</t>
-        </is>
-      </c>
-      <c r="O126" t="inlineStr">
-        <is>
-          <t>Integrated Bioelectronic and Optogenetic Methods to Study Brain-Body Circuits (2024)</t>
-        </is>
-      </c>
+          <t>Systematic Review and Meta-Analysis of Bilateral Centromedian Nucleus Neuromodulation for Multifocal and Generalized Epilepsy. (2025)</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr"/>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R126" t="inlineStr"/>
@@ -22269,12 +22261,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Neurological Surgery</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Rongze Lu</t>
+          <t>Min Kang</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -22299,7 +22291,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Brain tumor immune evasion mechanisms and chromatin programs in glioblastoma.</t>
+          <t>Multidisciplinary care and clinical trials in myasthenia gravis.</t>
         </is>
       </c>
       <c r="J127" t="inlineStr"/>
@@ -22307,27 +22299,19 @@
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/317918332</t>
-        </is>
-      </c>
-      <c r="N127" t="inlineStr">
-        <is>
-          <t>Protein phosphatase 2A regulates senescence and immunogenicity in medulloblastoma models (2026)</t>
-        </is>
-      </c>
-      <c r="O127" t="inlineStr">
-        <is>
-          <t>Tumor-intrinsic chromatin programs enforce immune evasion in glioblastoma (2026)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/181165</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
         <is>
-          <t>Advances in the understanding and therapeutic manipulation of cancer immune responsiveness: a Society for Immunotherapy of Cancer (SITC) review (2025) | Co-evolution of glioma and immune microenvironment (2024)</t>
+          <t>Optimising well-being in myasthenia gravis: a multidisciplinary approach (2026) | Switching to subcutaneous zilucoplan from intravenous complement component 5 inhibitors in generalised myasthenia gravis: a phase IIIb, open-label study (2025)</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R127" t="inlineStr"/>
@@ -22353,24 +22337,16 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Neuroscience Graduate Program (faculty)</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Sara Chung</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Assistant Professor</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
+          <t>Qili Liu</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>C</t>
@@ -22383,31 +22359,23 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Developmental psychology: parenting, ADHD and stress in Asian American college students.</t>
+          <t>Fly neurobiology of nutrient-specific appetite (wet lab)</t>
         </is>
       </c>
       <c r="J128" t="inlineStr"/>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr">
-        <is>
-          <t>https://researcherprofiles.org/profile/171132582</t>
-        </is>
-      </c>
-      <c r="N128" t="inlineStr">
-        <is>
-          <t>Parsing Day-to-Day Dynamics of ADHD and Perceived Stress in College Students: An Ecological Momentary Assessment Study (2026)</t>
-        </is>
-      </c>
-      <c r="O128" t="inlineStr">
-        <is>
-          <t>ADHD Knowledge as a Barrier to Problem Recognition in Asian American and Native Hawaiian/Pacific Islander Versus White College Students (2026)</t>
-        </is>
-      </c>
-      <c r="P128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
+      <c r="P128" t="inlineStr">
+        <is>
+          <t>Targeted cravings: Unraveling the drivers of nutrient-specific appetite (2025) | Opposing GPCR signaling programs protein intake setpoint in Drosophila (2024)</t>
+        </is>
+      </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
+          <t>https://neurograd.ucsf.edu/faculty</t>
         </is>
       </c>
       <c r="R128" t="inlineStr"/>
@@ -22429,17 +22397,17 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Psychiatry</t>
+          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only); Neurological Surgery; Neuroscience Graduate Program (faculty)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Selena Chan</t>
+          <t>Ritchie Chen</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Asst Professor In Residence</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -22459,7 +22427,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Psychiatry; community care programs, clinical and wellness work.</t>
+          <t>Engineers genetically targeted bioelectronic and optogenetic tools to map and control brain-body circuits.</t>
         </is>
       </c>
       <c r="J129" t="inlineStr"/>
@@ -22467,15 +22435,19 @@
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/174541</t>
+          <t>https://bms.ucsf.edu/people/ritchie-chen-phd-msc-bs</t>
         </is>
       </c>
       <c r="N129" t="inlineStr"/>
       <c r="O129" t="inlineStr"/>
-      <c r="P129" t="inlineStr"/>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>Interoceptive modulation of emotions (2025) | Integrated Bioelectronic and Optogenetic Methods to Study Brain-Body Circuits (2024)</t>
+        </is>
+      </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
+          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=4</t>
         </is>
       </c>
       <c r="R129" t="inlineStr"/>
@@ -22497,22 +22469,22 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Neurological Surgery</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Sharon Chiang</t>
+          <t>Rongze Lu</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -22527,7 +22499,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Quality-of-life outcome sets and vagus nerve stimulation outcomes in drug-resistant epilepsy.</t>
+          <t>Brain tumor immune evasion mechanisms and chromatin programs in glioblastoma.</t>
         </is>
       </c>
       <c r="J130" t="inlineStr"/>
@@ -22535,23 +22507,27 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/14718920</t>
+          <t>https://researcherprofiles.org/profile/317918332</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>Integrating longitudinal seizure, medication, and quality of life data into epilepsy eare: A randomized crossover study of an Epic-integrated dashboard (2026)</t>
+          <t>Protein phosphatase 2A regulates senescence and immunogenicity in medulloblastoma models (2026)</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>Influences of electrode density on intracranial seizure localisation: a single-blinded randomised crossover study (2025)</t>
-        </is>
-      </c>
-      <c r="P130" t="inlineStr"/>
+          <t>Tumor-intrinsic chromatin programs enforce immune evasion in glioblastoma (2026)</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>Advances in the understanding and therapeutic manipulation of cancer immune responsiveness: a Society for Immunotherapy of Cancer (SITC) review (2025) | Co-evolution of glioma and immune microenvironment (2024)</t>
+        </is>
+      </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
         </is>
       </c>
       <c r="R130" t="inlineStr"/>
@@ -22560,7 +22536,11 @@
       <c r="U130" t="inlineStr"/>
       <c r="V130" t="inlineStr"/>
       <c r="W130" t="inlineStr"/>
-      <c r="X130" t="inlineStr"/>
+      <c r="X130" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -22573,22 +22553,22 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Shinn-Huey Chou</t>
+          <t>Sara Chung</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -22603,7 +22583,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Breast imaging radiologist focused on high-risk screening and radiology training.</t>
+          <t>Developmental psychology: parenting, ADHD and stress in Asian American college students.</t>
         </is>
       </c>
       <c r="J131" t="inlineStr"/>
@@ -22611,19 +22591,23 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/540198469</t>
+          <t>https://researcherprofiles.org/profile/171132582</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>The parenthood journey in radiology: Challenges and opportunities (2025)</t>
-        </is>
-      </c>
-      <c r="O131" t="inlineStr"/>
+          <t>Parsing Day-to-Day Dynamics of ADHD and Perceived Stress in College Students: An Ecological Momentary Assessment Study (2026)</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>ADHD Knowledge as a Barrier to Problem Recognition in Asian American and Native Hawaiian/Pacific Islander Versus White College Students (2026)</t>
+        </is>
+      </c>
       <c r="P131" t="inlineStr"/>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
         </is>
       </c>
       <c r="R131" t="inlineStr"/>
@@ -22632,11 +22616,7 @@
       <c r="U131" t="inlineStr"/>
       <c r="V131" t="inlineStr"/>
       <c r="W131" t="inlineStr"/>
-      <c r="X131" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -22654,7 +22634,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Stephen Leung</t>
+          <t>Selena Chan</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -22679,7 +22659,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Benzodiazepine tapering recommendations for inpatient and residential care.</t>
+          <t>Psychiatry; community care programs, clinical and wellness work.</t>
         </is>
       </c>
       <c r="J132" t="inlineStr"/>
@@ -22687,14 +22667,10 @@
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/506961717</t>
-        </is>
-      </c>
-      <c r="N132" t="inlineStr">
-        <is>
-          <t>Toward clarifying ASAM's inpatient and residential benzodiazepine tapering recommendations (2026)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/174541</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr"/>
       <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr"/>
       <c r="Q132" t="inlineStr">
@@ -22721,22 +22697,22 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Neurological Surgery</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Sze Chun Winson Ho</t>
+          <t>Sharon Chiang</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -22751,7 +22727,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Pediatric neurosurgery and PP2A-targeted immunotherapy for brain tumors.</t>
+          <t>Quality-of-life outcome sets and vagus nerve stimulation outcomes in drug-resistant epilepsy.</t>
         </is>
       </c>
       <c r="J133" t="inlineStr"/>
@@ -22759,15 +22735,23 @@
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/325717114</t>
-        </is>
-      </c>
-      <c r="N133" t="inlineStr"/>
-      <c r="O133" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/14718920</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>Integrating longitudinal seizure, medication, and quality of life data into epilepsy eare: A randomized crossover study of an Epic-integrated dashboard (2026)</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Influences of electrode density on intracranial seizure localisation: a single-blinded randomised crossover study (2025)</t>
+        </is>
+      </c>
       <c r="P133" t="inlineStr"/>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R133" t="inlineStr"/>
@@ -22776,11 +22760,7 @@
       <c r="U133" t="inlineStr"/>
       <c r="V133" t="inlineStr"/>
       <c r="W133" t="inlineStr"/>
-      <c r="X133" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -22793,16 +22773,24 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Quantitative Biosciences Institute (home dept: Medicine)</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Terrelea Wong</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
+          <t>Shinn-Huey Chou</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>associate</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
           <t>C</t>
@@ -22815,7 +22803,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Card has no research text or papers.</t>
+          <t>Breast imaging radiologist focused on high-risk screening and radiology training.</t>
         </is>
       </c>
       <c r="J134" t="inlineStr"/>
@@ -22823,36 +22811,32 @@
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/terrelea.wong</t>
-        </is>
-      </c>
-      <c r="N134" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/540198469</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>The parenthood journey in radiology: Challenges and opportunities (2025)</t>
+        </is>
+      </c>
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr"/>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>https://qbi.ucsf.edu/investigators</t>
-        </is>
-      </c>
-      <c r="R134" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="S134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unspecified: </t>
-        </is>
-      </c>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr"/>
+      <c r="S134" t="inlineStr"/>
       <c r="T134" t="inlineStr"/>
       <c r="U134" t="inlineStr"/>
       <c r="V134" t="inlineStr"/>
-      <c r="W134" t="inlineStr">
-        <is>
-          <t>Search snippet (unfetched; profile 404s via fetch) indicates volunteer clinical professor in Medicine, not a PI; No research text</t>
-        </is>
-      </c>
-      <c r="X134" t="inlineStr"/>
+      <c r="W134" t="inlineStr"/>
+      <c r="X134" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -22870,7 +22854,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Tianyi Zhang</t>
+          <t>Stephen Leung</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -22895,7 +22879,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Elder financial exploitation in the digital age.</t>
+          <t>Benzodiazepine tapering recommendations for inpatient and residential care.</t>
         </is>
       </c>
       <c r="J135" t="inlineStr"/>
@@ -22903,12 +22887,12 @@
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/173787</t>
+          <t>https://researcherprofiles.org/profile/506961717</t>
         </is>
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>Elder Financial Exploitation in the Digital Age (2023)</t>
+          <t>Toward clarifying ASAM's inpatient and residential benzodiazepine tapering recommendations (2026)</t>
         </is>
       </c>
       <c r="O135" t="inlineStr"/>
@@ -22937,12 +22921,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>Neurological Surgery</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Virgina Lee</t>
+          <t>Sze Chun Winson Ho</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -22967,7 +22951,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Genetic variants in SNAP25 and OTUD6B in developmental and epileptic disorders.</t>
+          <t>Pediatric neurosurgery and PP2A-targeted immunotherapy for brain tumors.</t>
         </is>
       </c>
       <c r="J136" t="inlineStr"/>
@@ -22975,19 +22959,15 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/31165493</t>
-        </is>
-      </c>
-      <c r="N136" t="inlineStr">
-        <is>
-          <t>Biallelic OTUD6B variants associated with a Kabuki syndrome‐like disorder in three siblings: A clinical report and literature review (2024)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/325717114</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr"/>
       <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr"/>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurological Surgery)</t>
         </is>
       </c>
       <c r="R136" t="inlineStr"/>
@@ -23013,24 +22993,16 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Quantitative Biosciences Institute (home dept: Medicine)</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Weiya Mu</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>Assistant Professor</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
+          <t>Terrelea Wong</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
         <is>
           <t>C</t>
@@ -23043,7 +23015,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Radiology faculty; clinical neuroradiology and imaging anatomy, traumatic brain injury research; no ML described.</t>
+          <t>Card has no research text or papers.</t>
         </is>
       </c>
       <c r="J137" t="inlineStr"/>
@@ -23051,7 +23023,7 @@
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/416657849</t>
+          <t>https://profiles.ucsf.edu/terrelea.wong</t>
         </is>
       </c>
       <c r="N137" t="inlineStr"/>
@@ -23059,15 +23031,27 @@
       <c r="P137" t="inlineStr"/>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
-        </is>
-      </c>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
+          <t>https://qbi.ucsf.edu/investigators</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unspecified: </t>
+        </is>
+      </c>
       <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr"/>
       <c r="V137" t="inlineStr"/>
-      <c r="W137" t="inlineStr"/>
+      <c r="W137" t="inlineStr">
+        <is>
+          <t>Search snippet (unfetched; profile 404s via fetch) indicates volunteer clinical professor in Medicine, not a PI; No research text</t>
+        </is>
+      </c>
       <c r="X137" t="inlineStr"/>
     </row>
     <row r="138">
@@ -23081,12 +23065,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only)</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Wendy Yue</t>
+          <t>Tianyi Zhang</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -23111,7 +23095,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Spinal ependymal cell proliferation and opioid signalling.</t>
+          <t>Elder financial exploitation in the digital age.</t>
         </is>
       </c>
       <c r="J138" t="inlineStr"/>
@@ -23119,19 +23103,19 @@
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
-          <t>https://bms.ucsf.edu/people/wendy-yue-phd</t>
-        </is>
-      </c>
-      <c r="N138" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/173787</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>Elder Financial Exploitation in the Digital Age (2023)</t>
+        </is>
+      </c>
       <c r="O138" t="inlineStr"/>
-      <c r="P138" t="inlineStr">
-        <is>
-          <t>Endogenous opioid signalling regulates spinal ependymal cell proliferation (2024)</t>
-        </is>
-      </c>
+      <c r="P138" t="inlineStr"/>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=26</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Psychiatry)</t>
         </is>
       </c>
       <c r="R138" t="inlineStr"/>
@@ -23153,22 +23137,22 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Xiao Wu</t>
+          <t>Virgina Lee</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -23183,7 +23167,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Interventional radiology; cryoablation cost-effectiveness and radioembolization outcomes.</t>
+          <t>Genetic variants in SNAP25 and OTUD6B in developmental and epileptic disorders.</t>
         </is>
       </c>
       <c r="J139" t="inlineStr"/>
@@ -23191,23 +23175,19 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/115272775</t>
+          <t>https://researcherprofiles.org/profile/31165493</t>
         </is>
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>Cryoablation Versus Breast-Conserving Surgery for Early-Stage, Low-Risk Breast Cancer ≤ 1.5 cm: A Cost-Effectiveness Analysis (2026)</t>
+          <t>Biallelic OTUD6B variants associated with a Kabuki syndrome‐like disorder in three siblings: A clinical report and literature review (2024)</t>
         </is>
       </c>
       <c r="O139" t="inlineStr"/>
-      <c r="P139" t="inlineStr">
-        <is>
-          <t>Radioembolization for Colorectal Liver Metastases: Indications and Outcomes (2026) | Transarterial Embolization Versus Manipulation Under Anesthesia and Arthroscopic Capsular Release for Refractory Adhesive Capsulitis-A Cost-Effectiveness Analysis (2026)</t>
-        </is>
-      </c>
+      <c r="P139" t="inlineStr"/>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Neurology)</t>
         </is>
       </c>
       <c r="R139" t="inlineStr"/>
@@ -23216,7 +23196,11 @@
       <c r="U139" t="inlineStr"/>
       <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr"/>
-      <c r="X139" t="inlineStr"/>
+      <c r="X139" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -23234,17 +23218,17 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Xin Cynthia Wu</t>
+          <t>Weiya Mu</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -23259,7 +23243,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Head and neck imaging radiologist; clinical outcome studies with pembrolizumab.</t>
+          <t>Radiology faculty; clinical neuroradiology and imaging anatomy, traumatic brain injury research; no ML described.</t>
         </is>
       </c>
       <c r="J140" t="inlineStr"/>
@@ -23267,19 +23251,11 @@
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/319885332</t>
-        </is>
-      </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t>Statin Use Is Associated With Progression-Free Survival for Recurrent/Metastatic Head and Neck Squamous Cell Carcinoma Treated With Pembrolizumab (2026)</t>
-        </is>
-      </c>
-      <c r="O140" t="inlineStr">
-        <is>
-          <t>Metastatic Lymph Node Status Is Associated With Progression-Free Survival in Oral Cavity Squamous Cell Carcinoma Treated With Pembrolizumab (2026)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/416657849</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr"/>
       <c r="Q140" t="inlineStr">
         <is>
@@ -23292,11 +23268,7 @@
       <c r="U140" t="inlineStr"/>
       <c r="V140" t="inlineStr"/>
       <c r="W140" t="inlineStr"/>
-      <c r="X140" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -23309,22 +23281,22 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Radiology and Biomedical Imaging</t>
+          <t>Biomedical Sciences (BMS) PhD program faculty (Wayback 2026-07 copy, pages 0-12 and 26 only); Neuroscience Graduate Program (faculty)</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Yi Li</t>
+          <t>Wendy Yue</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -23334,12 +23306,12 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>medical-AI</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Clinical neuroradiology; image processing and analysis for the ABCD neuroimaging study.</t>
+          <t>Spinal ependymal cell proliferation and opioid signalling.</t>
         </is>
       </c>
       <c r="J141" t="inlineStr"/>
@@ -23347,19 +23319,19 @@
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/176541</t>
+          <t>https://bms.ucsf.edu/people/wendy-yue-phd</t>
         </is>
       </c>
       <c r="N141" t="inlineStr"/>
       <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr">
         <is>
-          <t>Chiari malformation type 1 is associated with a smaller fourth ventricle volume - a multi-cohort replication study (2026)</t>
+          <t>Endogenous opioid signalling regulates spinal ependymal cell proliferation (2024)</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+          <t>https://web.archive.org/web/20260710111852/https://bms.ucsf.edu/faculty?page=26</t>
         </is>
       </c>
       <c r="R141" t="inlineStr"/>
@@ -23368,11 +23340,7 @@
       <c r="U141" t="inlineStr"/>
       <c r="V141" t="inlineStr"/>
       <c r="W141" t="inlineStr"/>
-      <c r="X141" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -23385,16 +23353,24 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Quantitative Biosciences Institute (home dept: Biochemistry &amp; Biophysics)</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Yifan  Cheng</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr"/>
-      <c r="F142" t="inlineStr"/>
+          <t>Xiao Wu</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
       <c r="G142" t="inlineStr">
         <is>
           <t>C</t>
@@ -23407,7 +23383,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Structural biology and cryo-EM.</t>
+          <t>Interventional radiology; cryoablation cost-effectiveness and radioembolization outcomes.</t>
         </is>
       </c>
       <c r="J142" t="inlineStr"/>
@@ -23415,19 +23391,23 @@
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
-          <t>https://cryoem.ucsf.edu</t>
-        </is>
-      </c>
-      <c r="N142" t="inlineStr"/>
+          <t>https://researcherprofiles.org/profile/115272775</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>Cryoablation Versus Breast-Conserving Surgery for Early-Stage, Low-Risk Breast Cancer ≤ 1.5 cm: A Cost-Effectiveness Analysis (2026)</t>
+        </is>
+      </c>
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
         <is>
-          <t>Structural energetics of cold sensitivity (2026) | Antibody reveals conformational latch regulating dimerization in β- and γ-herpesvirus proteases (2026)</t>
+          <t>Radioembolization for Colorectal Liver Metastases: Indications and Outcomes (2026) | Transarterial Embolization Versus Manipulation Under Anesthesia and Arthroscopic Capsular Release for Refractory Adhesive Capsulitis-A Cost-Effectiveness Analysis (2026)</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>https://qbi.ucsf.edu/investigators</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R142" t="inlineStr"/>
@@ -23454,7 +23434,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Yoo Jin Lee</t>
+          <t>Xin Cynthia Wu</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -23474,12 +23454,12 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>medical-AI</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Clinical thoracic/cardiac radiology; MRI image quality studies, some AI-assisted segmentation.</t>
+          <t>Head and neck imaging radiologist; clinical outcome studies with pembrolizumab.</t>
         </is>
       </c>
       <c r="J143" t="inlineStr"/>
@@ -23487,16 +23467,20 @@
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
-          <t>https://researcherprofiles.org/profile/159721860</t>
-        </is>
-      </c>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
-      <c r="P143" t="inlineStr">
-        <is>
-          <t>Determinants of image quality in respiratory triggered free breathing lung MRI at 0.55 T in adults (2026) | AI-Assisted segmentation and volumetric reconstruction of radiographs through multi-angular scintillation imaging (2026)</t>
-        </is>
-      </c>
+          <t>https://researcherprofiles.org/profile/319885332</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Statin Use Is Associated With Progression-Free Survival for Recurrent/Metastatic Head and Neck Squamous Cell Carcinoma Treated With Pembrolizumab (2026)</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Metastatic Lymph Node Status Is Associated With Progression-Free Survival in Oral Cavity Squamous Cell Carcinoma Treated With Pembrolizumab (2026)</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr"/>
       <c r="Q143" t="inlineStr">
         <is>
           <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
@@ -23520,29 +23504,21 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Neuroscience Graduate Program (faculty)</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Bob X. Wang</t>
-        </is>
-      </c>
-      <c r="E144" t="inlineStr">
-        <is>
-          <t>Associate Professor of Instruction</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr">
-        <is>
-          <t>associate</t>
-        </is>
-      </c>
+          <t>Xin Duan</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
           <t>C</t>
@@ -23555,31 +23531,23 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Biosphere-atmosphere interactions, carbon and hydrological cycles; teaching-track chemistry.</t>
+          <t>Molecular and genetic assembly of neural circuits, optic neuropathy (wet lab)</t>
         </is>
       </c>
       <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>wangx@usf.edu</t>
-        </is>
-      </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/wang.aspx</t>
-        </is>
-      </c>
-      <c r="M144" t="inlineStr">
-        <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/wang.aspx</t>
-        </is>
-      </c>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
       <c r="N144" t="inlineStr"/>
       <c r="O144" t="inlineStr"/>
-      <c r="P144" t="inlineStr"/>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>Cell-intrinsic vulnerability and immune activation cooperate to drive degeneration in a mitochondrial complex I deficiency model of optic neuropathy (2026) | Molecular and cellular dynamics of the developing human neocortex (2025)</t>
+        </is>
+      </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
+          <t>https://neurograd.ucsf.edu/faculty</t>
         </is>
       </c>
       <c r="R144" t="inlineStr"/>
@@ -23588,11 +23556,7 @@
       <c r="U144" t="inlineStr"/>
       <c r="V144" t="inlineStr"/>
       <c r="W144" t="inlineStr"/>
-      <c r="X144" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -23600,22 +23564,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Christian Tang</t>
+          <t>Yi Li</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Associate Professor of Instruction</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -23630,52 +23594,40 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>No research text or papers on the card.</t>
+          <t>Clinical neuroradiology; image processing and analysis for the ABCD neuroimaging study.</t>
         </is>
       </c>
       <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>ctang3@usf.edu</t>
-        </is>
-      </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
-        </is>
-      </c>
-      <c r="M145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>https://researcherprofiles.org/profile/176541</t>
+        </is>
+      </c>
       <c r="N145" t="inlineStr"/>
       <c r="O145" t="inlineStr"/>
-      <c r="P145" t="inlineStr"/>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>Chiari malformation type 1 is associated with a smaller fourth ventricle volume - a multi-cohort replication study (2026)</t>
+        </is>
+      </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
-        </is>
-      </c>
-      <c r="R145" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="S145" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Unspecified: </t>
-        </is>
-      </c>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr"/>
+      <c r="S145" t="inlineStr"/>
       <c r="T145" t="inlineStr"/>
       <c r="U145" t="inlineStr"/>
       <c r="V145" t="inlineStr"/>
-      <c r="W145" t="inlineStr">
-        <is>
-          <t>teaching faculty, not a PI; not ML</t>
-        </is>
-      </c>
+      <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr">
         <is>
           <t>associate: confirm promoted 2020+</t>
@@ -23688,29 +23640,21 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Quantitative Biosciences Institute (home dept: Biochemistry &amp; Biophysics)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Jin Jia</t>
-        </is>
-      </c>
-      <c r="E146" t="inlineStr">
-        <is>
-          <t>Assistant Professor</t>
-        </is>
-      </c>
-      <c r="F146" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
+          <t>Yifan  Cheng</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
           <t>C</t>
@@ -23723,31 +23667,27 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Chemistry department; no research text, presumed chemistry lab.</t>
+          <t>Structural biology and cryo-EM.</t>
         </is>
       </c>
       <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>jinjia@usf.edu</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/jia.aspx</t>
-        </is>
-      </c>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/jia.aspx</t>
+          <t>https://cryoem.ucsf.edu</t>
         </is>
       </c>
       <c r="N146" t="inlineStr"/>
       <c r="O146" t="inlineStr"/>
-      <c r="P146" t="inlineStr"/>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>Structural energetics of cold sensitivity (2026) | Antibody reveals conformational latch regulating dimerization in β- and γ-herpesvirus proteases (2026)</t>
+        </is>
+      </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
+          <t>https://qbi.ucsf.edu/investigators</t>
         </is>
       </c>
       <c r="R146" t="inlineStr"/>
@@ -23764,27 +23704,27 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Molecular Pharmacology and Physiology</t>
+          <t>Radiology and Biomedical Imaging</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Lei Wang</t>
+          <t>Yoo Jin Lee</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -23794,40 +23734,32 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>medical-AI</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Blood pressure and renal function physiology; kidney injury and transplantation mechanisms.</t>
+          <t>Clinical thoracic/cardiac radiology; MRI image quality studies, some AI-assisted segmentation.</t>
         </is>
       </c>
       <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>leiwang@usf.edu</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/leiwang</t>
-        </is>
-      </c>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/leiwang</t>
+          <t>https://researcherprofiles.org/profile/159721860</t>
         </is>
       </c>
       <c r="N147" t="inlineStr"/>
       <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr">
         <is>
-          <t>Limb Ischemia-Reperfusion Injury in Rats is partially mediated by enhancing Necroptosis via Phosphorylation of RIPK1 and MLKL (2026) | Glomerulus-targeted nanotherapy via collagen IV-α3 binding enhances renal immunoregulation in lupus nephritis (2026)</t>
+          <t>Determinants of image quality in respiratory triggered free breathing lung MRI at 0.55 T in adults (2026) | AI-Assisted segmentation and volumetric reconstruction of radiographs through multi-angular scintillation imaging (2026)</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Radiology)</t>
         </is>
       </c>
       <c r="R147" t="inlineStr"/>
@@ -23836,7 +23768,11 @@
       <c r="U147" t="inlineStr"/>
       <c r="V147" t="inlineStr"/>
       <c r="W147" t="inlineStr"/>
-      <c r="X147" t="inlineStr"/>
+      <c r="X147" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -23849,22 +23785,22 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Chemical, Biological and Materials Engineering</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Weizhong Zou</t>
+          <t>Bob X. Wang</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor of Instruction</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -23879,43 +23815,31 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Polymer and materials engineering with multiscale modelling and data-driven tools.</t>
+          <t>Biosphere-atmosphere interactions, carbon and hydrological cycles; teaching-track chemistry.</t>
         </is>
       </c>
       <c r="J148" t="inlineStr"/>
       <c r="K148" t="inlineStr">
         <is>
-          <t>wzou@usf.edu</t>
+          <t>wangx@usf.edu</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/engineering/chbme/people/zou.aspx</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/wang.aspx</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>https://thezoulab.com/</t>
-        </is>
-      </c>
-      <c r="N148" t="inlineStr">
-        <is>
-          <t>Real-Time Quantification of Molecular-Level Dynamic Behaviors Underpinning Shear Thinning in End-Linked Associative Polymer Networks (2024)</t>
-        </is>
-      </c>
-      <c r="O148" t="inlineStr">
-        <is>
-          <t>Toughening and Imparting Deconstructability to 3D-Printed Glassy Thermosets with "Transferinker" Additives (2024)</t>
-        </is>
-      </c>
-      <c r="P148" t="inlineStr">
-        <is>
-          <t>Addition to: "Toughening and Imparting Deconstructability to 3D-Printed Glassy Thermosets with "Transferinker" Additives" (2025)</t>
-        </is>
-      </c>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/wang.aspx</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="inlineStr"/>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/engineering/chbme/people/index.aspx</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
         </is>
       </c>
       <c r="R148" t="inlineStr"/>
@@ -23924,7 +23848,11 @@
       <c r="U148" t="inlineStr"/>
       <c r="V148" t="inlineStr"/>
       <c r="W148" t="inlineStr"/>
-      <c r="X148" t="inlineStr"/>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -23942,12 +23870,12 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Wenqi (Vince) Liu</t>
+          <t>Christian Tang</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Associate Professor of Instruction</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -23967,43 +23895,47 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Host-guest chemistry for sensing, catalysis and separations; functional molecular materials.</t>
+          <t>No research text or papers on the card.</t>
         </is>
       </c>
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr">
         <is>
-          <t>wenqi@usf.edu</t>
+          <t>ctang3@usf.edu</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>https://nam04.safelinks.protection.outlook.com/?url=http%3A%2F%2Fwww.vincentchemistry.com%2F&amp;data=04%7C01%7Cpaigeromero%40usf.edu%7C27a9b8f622b44829bb3908d96d88e19d%7C741bf7dee2e546df8d6782607df9deaa%7C0%7C0%7C637661256924716608%7CUnknown%7CTWFpbGZsb3d8eyJWIjoiMC4wLjAwMDAiLCJQIjoiV2luMzIiLCJBTiI6Ik1haWwiLCJXVCI6Mn0%3D%7C1000&amp;sdata=mbuJDqqgQC2eHi%2FxUp%2BM4dMT2Zde%2FpwxCJtcyUDXB4g%3D&amp;reserved=0</t>
-        </is>
-      </c>
-      <c r="M149" t="inlineStr">
-        <is>
-          <t>https://nam04.safelinks.protection.outlook.com/?url=http%3A%2F%2Fwww.vincentchemistry.com%2F&amp;data=04%7C01%7Cpaigeromero%40usf.edu%7C27a9b8f622b44829bb3908d96d88e19d%7C741bf7dee2e546df8d6782607df9deaa%7C0%7C0%7C637661256924716608%7CUnknown%7CTWFpbGZsb3d8eyJWIjoiMC4wLjAwMDAiLCJQIjoiV2luMzIiLCJBTiI6Ik1haWwiLCJXVCI6Mn0%3D%7C1000&amp;sdata=mbuJDqqgQC2eHi%2FxUp%2BM4dMT2Zde%2FpwxCJtcyUDXB4g%3D&amp;reserved=0</t>
-        </is>
-      </c>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
       <c r="O149" t="inlineStr"/>
-      <c r="P149" t="inlineStr">
-        <is>
-          <t>Mechanically Planar Chiral Molecules by a SuFEx-Auxiliary Approach (2026) | Oxonium-Embedded Benzo[&amp;lt;i&amp;gt;b&amp;lt;/i&amp;gt;]perylene: A Redox-Switchable Closed-Shell π‑Cation, and Its Paramagnetic Charge-Transfer Salt with TCNE&amp;lt;sup&amp;gt;•&amp;lt;/sup&amp;gt; (2026)</t>
-        </is>
-      </c>
+      <c r="P149" t="inlineStr"/>
       <c r="Q149" t="inlineStr">
         <is>
           <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
         </is>
       </c>
-      <c r="R149" t="inlineStr"/>
-      <c r="S149" t="inlineStr"/>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unspecified: </t>
+        </is>
+      </c>
       <c r="T149" t="inlineStr"/>
       <c r="U149" t="inlineStr"/>
       <c r="V149" t="inlineStr"/>
-      <c r="W149" t="inlineStr"/>
+      <c r="W149" t="inlineStr">
+        <is>
+          <t>teaching faculty, not a PI; not ML</t>
+        </is>
+      </c>
       <c r="X149" t="inlineStr">
         <is>
           <t>associate: confirm promoted 2020+</t>
@@ -24021,12 +23953,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Molecular Medicine</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Xuewei Wang</t>
+          <t>Jin Jia</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
@@ -24051,23 +23983,23 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Neuroregeneration and neuroprotection; axon regeneration wet-lab biology.</t>
+          <t>Chemistry department; no research text, presumed chemistry lab.</t>
         </is>
       </c>
       <c r="J150" t="inlineStr"/>
       <c r="K150" t="inlineStr">
         <is>
-          <t>xueweiwang@usf.edu</t>
+          <t>jinjia@usf.edu</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/molecularmedicine/faculty/xueweiwang</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/jia.aspx</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
         <is>
-          <t>https://cloud.usf.edu/FacultyDirectory/api/get/profile/xueweiwang/document/cv</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/jia.aspx</t>
         </is>
       </c>
       <c r="N150" t="inlineStr"/>
@@ -24075,7 +24007,7 @@
       <c r="P150" t="inlineStr"/>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/molecularmedicine/faculty/</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
         </is>
       </c>
       <c r="R150" t="inlineStr"/>
@@ -24097,12 +24029,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Molecular Pharmacology and Physiology</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Ying Wang</t>
+          <t>Lei Wang</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -24127,31 +24059,35 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Chemistry education research on student affect and learning.</t>
+          <t>Blood pressure and renal function physiology; kidney injury and transplantation mechanisms.</t>
         </is>
       </c>
       <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr">
         <is>
-          <t>yingw@usf.edu</t>
+          <t>leiwang@usf.edu</t>
         </is>
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/ying-wang.aspx</t>
+          <t>https://health.usf.edu/medicine/mpp/faculty/leiwang</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>https://sites.google.com/view/wang-research-group/home</t>
+          <t>https://health.usf.edu/medicine/mpp/faculty/leiwang</t>
         </is>
       </c>
       <c r="N151" t="inlineStr"/>
       <c r="O151" t="inlineStr"/>
-      <c r="P151" t="inlineStr"/>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>Limb Ischemia-Reperfusion Injury in Rats is partially mediated by enhancing Necroptosis via Phosphorylation of RIPK1 and MLKL (2026) | Glomerulus-targeted nanotherapy via collagen IV-α3 binding enhances renal immunoregulation in lupus nephritis (2026)</t>
+        </is>
+      </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
+          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
         </is>
       </c>
       <c r="R151" t="inlineStr"/>
@@ -24173,22 +24109,22 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Molecular Pharmacology and Physiology</t>
+          <t>Chemical, Biological and Materials Engineering</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Ying Yang</t>
+          <t>Weizhong Zou</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Associate Professor</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -24203,35 +24139,43 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Lymphatic vasculature biology and lymphatic valve molecular mechanisms.</t>
+          <t>Polymer and materials engineering with multiscale modelling and data-driven tools.</t>
         </is>
       </c>
       <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
-          <t>yingyang@usf.edu</t>
+          <t>wzou@usf.edu</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/yingyang</t>
+          <t>https://www.usf.edu/engineering/chbme/people/zou.aspx</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/yingyang</t>
-        </is>
-      </c>
-      <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr"/>
+          <t>https://thezoulab.com/</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>Real-Time Quantification of Molecular-Level Dynamic Behaviors Underpinning Shear Thinning in End-Linked Associative Polymer Networks (2024)</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Toughening and Imparting Deconstructability to 3D-Printed Glassy Thermosets with "Transferinker" Additives (2024)</t>
+        </is>
+      </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>Lymphatic Malformations With Activating KRAS Mutations Impair Lymphatic Valve Development Through Matrix Metalloproteinases (2026) | Rictor, an mTORC2 Protein, Regulates Murine Lymphatic Valve Formation Through the AKT-FOXO1 Signaling (2024)</t>
+          <t>Addition to: "Toughening and Imparting Deconstructability to 3D-Printed Glassy Thermosets with "Transferinker" Additives" (2025)</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
+          <t>https://www.usf.edu/engineering/chbme/people/index.aspx</t>
         </is>
       </c>
       <c r="R152" t="inlineStr"/>
@@ -24240,11 +24184,7 @@
       <c r="U152" t="inlineStr"/>
       <c r="V152" t="inlineStr"/>
       <c r="W152" t="inlineStr"/>
-      <c r="X152" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+</t>
-        </is>
-      </c>
+      <c r="X152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -24257,22 +24197,22 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Molecular Pharmacology and Physiology</t>
+          <t>Chemistry</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Yonggang Ma</t>
+          <t>Wenqi (Vince) Liu</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -24287,39 +24227,35 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Immune regulation of heart failure after myocardial infarction; cardiovascular biology.</t>
+          <t>Host-guest chemistry for sensing, catalysis and separations; functional molecular materials.</t>
         </is>
       </c>
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
-          <t>yma4@usf.edu</t>
+          <t>wenqi@usf.edu</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/yma4</t>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=http%3A%2F%2Fwww.vincentchemistry.com%2F&amp;data=04%7C01%7Cpaigeromero%40usf.edu%7C27a9b8f622b44829bb3908d96d88e19d%7C741bf7dee2e546df8d6782607df9deaa%7C0%7C0%7C637661256924716608%7CUnknown%7CTWFpbGZsb3d8eyJWIjoiMC4wLjAwMDAiLCJQIjoiV2luMzIiLCJBTiI6Ik1haWwiLCJXVCI6Mn0%3D%7C1000&amp;sdata=mbuJDqqgQC2eHi%2FxUp%2BM4dMT2Zde%2FpwxCJtcyUDXB4g%3D&amp;reserved=0</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/yma4</t>
-        </is>
-      </c>
-      <c r="N153" t="inlineStr">
-        <is>
-          <t>Glucocorticoids impair T lymphopoiesis after myocardial infarction (2024)</t>
-        </is>
-      </c>
+          <t>https://nam04.safelinks.protection.outlook.com/?url=http%3A%2F%2Fwww.vincentchemistry.com%2F&amp;data=04%7C01%7Cpaigeromero%40usf.edu%7C27a9b8f622b44829bb3908d96d88e19d%7C741bf7dee2e546df8d6782607df9deaa%7C0%7C0%7C637661256924716608%7CUnknown%7CTWFpbGZsb3d8eyJWIjoiMC4wLjAwMDAiLCJQIjoiV2luMzIiLCJBTiI6Ik1haWwiLCJXVCI6Mn0%3D%7C1000&amp;sdata=mbuJDqqgQC2eHi%2FxUp%2BM4dMT2Zde%2FpwxCJtcyUDXB4g%3D&amp;reserved=0</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr"/>
       <c r="O153" t="inlineStr"/>
       <c r="P153" t="inlineStr">
         <is>
-          <t>Aging diminishes thymic output, reduces naive T cells, promotes memory T-cell accumulation, and impairs thymic regeneration (2026) | Lung endothelial cell senescence impairs barrier function and promotes neutrophil adhesion and migration (2025)</t>
+          <t>Mechanically Planar Chiral Molecules by a SuFEx-Auxiliary Approach (2026) | Oxonium-Embedded Benzo[&amp;lt;i&amp;gt;b&amp;lt;/i&amp;gt;]perylene: A Redox-Switchable Closed-Shell π‑Cation, and Its Paramagnetic Charge-Transfer Salt with TCNE&amp;lt;sup&amp;gt;•&amp;lt;/sup&amp;gt; (2026)</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
         </is>
       </c>
       <c r="R153" t="inlineStr"/>
@@ -24328,7 +24264,331 @@
       <c r="U153" t="inlineStr"/>
       <c r="V153" t="inlineStr"/>
       <c r="W153" t="inlineStr"/>
-      <c r="X153" t="inlineStr"/>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>4</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>University of South Florida</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Molecular Medicine</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Xuewei Wang</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Neuroregeneration and neuroprotection; axon regeneration wet-lab biology.</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>xueweiwang@usf.edu</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/molecularmedicine/faculty/xueweiwang</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>https://cloud.usf.edu/FacultyDirectory/api/get/profile/xueweiwang/document/cv</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
+      <c r="P154" t="inlineStr"/>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/molecularmedicine/faculty/</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="inlineStr"/>
+      <c r="U154" t="inlineStr"/>
+      <c r="V154" t="inlineStr"/>
+      <c r="W154" t="inlineStr"/>
+      <c r="X154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>4</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>University of South Florida</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Ying Wang</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Chemistry education research on student affect and learning.</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>yingw@usf.edu</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/ying-wang.aspx</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/wang-research-group/home</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
+      <c r="P155" t="inlineStr"/>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>https://www.usf.edu/arts-sciences/departments/chemistry/faculty/index.aspx</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr"/>
+      <c r="S155" t="inlineStr"/>
+      <c r="T155" t="inlineStr"/>
+      <c r="U155" t="inlineStr"/>
+      <c r="V155" t="inlineStr"/>
+      <c r="W155" t="inlineStr"/>
+      <c r="X155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>4</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>University of South Florida</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Molecular Pharmacology and Physiology</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Ying Yang</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>associate</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Lymphatic vasculature biology and lymphatic valve molecular mechanisms.</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>yingyang@usf.edu</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/yingyang</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/yingyang</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>Lymphatic Malformations With Activating KRAS Mutations Impair Lymphatic Valve Development Through Matrix Metalloproteinases (2026) | Rictor, an mTORC2 Protein, Regulates Murine Lymphatic Valve Formation Through the AKT-FOXO1 Signaling (2024)</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
+        </is>
+      </c>
+      <c r="R156" t="inlineStr"/>
+      <c r="S156" t="inlineStr"/>
+      <c r="T156" t="inlineStr"/>
+      <c r="U156" t="inlineStr"/>
+      <c r="V156" t="inlineStr"/>
+      <c r="W156" t="inlineStr"/>
+      <c r="X156" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>4</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>University of South Florida</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Molecular Pharmacology and Physiology</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Yonggang Ma</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>assistant</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Immune regulation of heart failure after myocardial infarction; cardiovascular biology.</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>yma4@usf.edu</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/yma4</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/yma4</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>Glucocorticoids impair T lymphopoiesis after myocardial infarction (2024)</t>
+        </is>
+      </c>
+      <c r="O157" t="inlineStr"/>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>Aging diminishes thymic output, reduces naive T cells, promotes memory T-cell accumulation, and impairs thymic regeneration (2026) | Lung endothelial cell senescence impairs barrier function and promotes neutrophil adhesion and migration (2025)</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>https://health.usf.edu/medicine/mpp/faculty/</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr"/>
+      <c r="S157" t="inlineStr"/>
+      <c r="T157" t="inlineStr"/>
+      <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr"/>
+      <c r="W157" t="inlineStr"/>
+      <c r="X157" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24903,7 +25163,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>people 3 | need email 10 | check 17 | dropped C 47</t>
+          <t>people 3 | need email 10 | check 17 | dropped C 51</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -28046,7 +28306,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>blocked</t>
+          <t>done</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -28055,7 +28315,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0</v>
+        <v>99</v>
+      </c>
+      <c r="F79" t="n">
+        <v>99</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -28064,7 +28327,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>403 to our fetch (bot-blocked); not worked around. Program lists ~100 faculty; most are in Profiles depts (Neurology, Psychiatry, Biochem etc.) already rostered</t>
+          <t>bot-check blocked for us; page saved by the applicant in her own browser (data/snapshots/manual/ucsf-neurograd-faculty.pdf); 99 names parsed by code (~100 per catalog); titles from our UCSF Profiles rosters (66/99)</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>

</xml_diff>

<commit_message>
Neil Gong theme -> trustworthy-ML (coordinator correction)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SHXVUB5nxWZdDwRJd5MuyH
</commit_message>
<xml_diff>
--- a/data/export/batch1.xlsx
+++ b/data/export/batch1.xlsx
@@ -567,87 +567,91 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>University of California San Francisco</t>
+          <t>Duke University</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bioengineering and Therapeutic Sciences (Profiles dept Bioengineering)</t>
+          <t>Electrical &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brian Cheung</t>
+          <t>Neil Gong</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Associate Professor of Electrical and Computer Engineering</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>assistant</t>
+          <t>associate</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>trustworthy-ML</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>ICML 3, Trans. Mach. Learn. Res. 2, WACV 1, NeurIPS 1</t>
+          <t>NeurIPS 3, ICLR 2, ACL (1) 1, ACL (Findings) 1, EMNLP 1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>check which PhD program can admit (not a CS/Stat/DS dept)</t>
+          <t>AI-type dept: Electrical &amp; Computer Engineering</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Bioengineering and therapeutic sciences; no research text on card.</t>
+          <t>Zero-shot autonomous microscopy for scalable characterization of 2D materials.</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr">
         <is>
-          <t>bcheung@ucsf.edu</t>
+          <t>neil.gong@duke.edu</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>https://briancheung.github.io</t>
+          <t>https://ece.duke.edu/people/neil-gong/</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>https://discolab.org/</t>
+          <t>https://people.duke.edu/~zg70/index.html</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Words That Make Language Models Perceive</t>
+          <t>A Critical Evaluation of Defenses against Prompt Injection Attacks</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>What if Eye...? Computationally Recreating Vision Evolution</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr"/>
+          <t>Fingerprinting LLMs via Prompt Injection</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Zero-Shot Autonomous Microscopy for Scalable and Intelligent Characterization of 2D Materials (2025)</t>
+        </is>
+      </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>https://profiles.ucsf.edu/search/advanced (Department=Bioengineering)</t>
+          <t>https://ece.duke.edu/faculty</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -657,26 +661,26 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Yes: Open positions Postdocs, students, and research engineers interested in AI for science.</t>
+          <t>Yes: I am looking for postdocs, Ph.D. students, master's students, and undergraduate researchers. If you are interested in pursuing a Ph.D., please submit your application to Duke ECE.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>Contact Email: bcheung@ucsf.edu</t>
-        </is>
-      </c>
+      <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Convergent representations across modalities (Platonic Representation Hypothesis) connects to her BioCLIP+EfficientNet representation/evaluation work (arborphy) and probing/interpretability work (interp); AI for scientific discovery fits Bio-AI goal.</t>
+          <t>His work on evaluating prompt-injection defenses and secure agentic AI connects to my multi-agent system with verification and trust gating (agents).</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Input homepage was a UCSF Profiles page; true lab site is discolab.org; Dept is Bioengineering and Therapeutic Sciences (School of Pharmacy); doctoral program to apply through not stated (check BTS vs BMI); Lab described as 'post AGI' and 'Last updated: Oct 2026': very recently launched</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr"/>
+          <t>first-pass summary describes different work (microscopy of 2D materials); possibly wrong person/mismatch; warns he receives many emails and may not respond</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -684,17 +688,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>University of California San Francisco</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bellini College of AI, Cybersecurity and Computing</t>
+          <t>Bioengineering and Therapeutic Sciences (Profiles dept Bioengineering)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ning Wang</t>
+          <t>Brian Cheung</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -714,57 +718,57 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>trustworthy-ML</t>
+          <t>other</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>ACL (6) 1</t>
+          <t>ICML 3, Trans. Mach. Learn. Res. 2, WACV 1, NeurIPS 1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>AI-type dept: Bellini College of AI, Cybersecurity and Comp</t>
+          <t>check which PhD program can admit (not a CS/Stat/DS dept)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Federated learning, network intrusion detection, adversarial ML, differential privacy, LLMs in cybersecurity.</t>
+          <t>Bioengineering and therapeutic sciences; no research text on card.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>ningw@usf.edu</t>
+          <t>bcheung@ucsf.edu</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/ning-wang.aspx</t>
+          <t>https://briancheung.github.io</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>https://trust-ai-lab.github.io/index.html</t>
+          <t>https://discolab.org/</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Learning from Textual Radiology Reports: A Benchmark Dataset for Coronary CT Angiography</t>
+          <t>Words That Make Language Models Perceive</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>EarlyShield: Early-Stage Screening for Robust Personalized Federated Learning</t>
+          <t>What if Eye...? Computationally Recreating Vision Evolution</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/index.aspx</t>
+          <t>https://profiles.ucsf.edu/search/advanced (Department=Bioengineering)</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -774,26 +778,26 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Yes: Tasnimul Hossain Tomal joined SPRAI lab as a PhD student. (Aug. 2026; openings link on lab site not read)</t>
+          <t>Yes: Open positions Postdocs, students, and research engineers interested in AI for science.</t>
         </is>
       </c>
       <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Contact Email: bcheung@ucsf.edu</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>Agents/reliability and evaluation work connects loosely to trustworthy-AI security; federated medical imaging (Aegis) is the only bio link.</t>
+          <t>Convergent representations across modalities (Platonic Representation Hypothesis) connects to her BioCLIP+EfficientNet representation/evaluation work (arborphy) and probing/interpretability work (interp); AI for scientific discovery fits Bio-AI goal.</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>security-focused ML</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>dossier reader says B: Mostly AI security/privacy rather than core ML; in scope but weaker.; dossier recruiting: quote not on page, re-check</t>
-        </is>
-      </c>
+          <t>Input homepage was a UCSF Profiles page; true lab site is discolab.org; Dept is Bioengineering and Therapeutic Sciences (School of Pharmacy); doctoral program to apply through not stated (check BTS vs BMI); Lab described as 'post AGI' and 'Last updated: Oct 2026': very recently launched</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -801,17 +805,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Boston University</t>
+          <t>University of South Florida</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Psychological &amp; Brain Sciences; Graduate Program for Neuroscience (faculty); Center for Systems Neuroscience</t>
+          <t>Bellini College of AI, Cybersecurity and Computing</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Arthur Lee</t>
+          <t>Ning Wang</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -826,56 +830,62 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NeuroAI</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+          <t>trustworthy-ML</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ACL (6) 1</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>check which PhD program can admit (not a CS/Stat/DS dept)</t>
+          <t>AI-type dept: Bellini College of AI, Cybersecurity and Comp</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Card has no research text or papers.</t>
+          <t>Federated learning, network intrusion detection, adversarial ML, differential privacy, LLMs in cybersecurity.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>artlee@bu.edu</t>
+          <t>ningw@usf.edu</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>https://www.bu.edu/psych/profile/arthur-sangil-lee/</t>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/ning-wang.aspx</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>http://thedecodinglab.com/</t>
+          <t>https://trust-ai-lab.github.io/index.html</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Neural decoders: saving the baby from the bathwater</t>
+          <t>Learning from Textual Radiology Reports: A Benchmark Dataset for Coronary CT Angiography</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Distinguishing deception from its confounds by improving the validity of fMRI-based neural prediction</t>
+          <t>EarlyShield: Early-Stage Screening for Robust Personalized Federated Learning</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>https://www.bu.edu/psych/people/faculty/</t>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/index.aspx</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -885,28 +895,24 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>Yes: We are looking for Ph.D. students interested in our research.</t>
+          <t>Yes: Tasnimul Hossain Tomal joined SPRAI lab as a PhD student. (Aug. 2026; openings link on lab site not read)</t>
         </is>
       </c>
       <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Please feel free to send an email to Arthur (see contact) to let him know to look out for your application.</t>
-        </is>
-      </c>
+      <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>His interest in validating neural decoders (confounds, interpretability) connects to the EEG motor-imagery decoder with run-grouped validation.</t>
+          <t>Agents/reliability and evaluation work connects loosely to trustworthy-AI security; federated medical imaging (Aegis) is the only bio link.</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>psychology department; applications go through Psychology or Neuroscience program, not CS/Stats</t>
+          <t>security-focused ML</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>also listed as Arthur Sangil Lee</t>
+          <t>dossier reader says B: Mostly AI security/privacy rather than core ML; in scope but weaker.; dossier recruiting: quote not on page, re-check</t>
         </is>
       </c>
     </row>
@@ -916,17 +922,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cold Spring Harbor Laboratory</t>
+          <t>Boston University</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CSHL Faculty (Research)</t>
+          <t>Psychological &amp; Brain Sciences; Graduate Program for Neuroscience (faculty); Center for Systems Neuroscience</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Helen Hou</t>
+          <t>Arthur Lee</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -949,9 +955,7 @@
           <t>NeuroAI</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
@@ -960,43 +964,39 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Brain-body motor control; ML video analysis and neural encoding from behavior via Gaussian splatting.</t>
+          <t>Card has no research text or papers.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>hou@cshl.edu</t>
+          <t>artlee@bu.edu</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>https://www.cshl.edu/research/faculty-staff/helen-hou/</t>
+          <t>https://www.bu.edu/psych/profile/arthur-sangil-lee/</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>https://houlab.org</t>
+          <t>http://thedecodinglab.com/</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Cheese3D enables sensitive detection and analysis of whole-face movement in mice</t>
+          <t>Neural decoders: saving the baby from the bathwater</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>A generic noninvasive neuromotor interface for human-computer interaction</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>A case study on the use of end-to-end real-time monitoring to ensure quality of oral solid dosage forms in pharmaceutical development. (2025) | Chemical genetic screens reveal defective lysosomal trafficking as synthetic lethal with NF1 loss (2024)</t>
-        </is>
-      </c>
+          <t>Distinguishing deception from its confounds by improving the validity of fMRI-based neural prediction</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>https://www.cshl.edu/research/faculty-staff/</t>
+          <t>https://www.bu.edu/psych/people/faculty/</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1006,24 +1006,28 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>Yes: We are actively recruiting at all levels, including but not limited to Students, Postdocs, and Research Technicians.</t>
+          <t>Yes: We are looking for Ph.D. students interested in our research.</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr">
         <is>
-          <t>Please get in touch via hou [at] cshl.edu and include your CV/resume and contact information of three references. (IMPORTANT: Please include the term #hou_lab _ candidate somewhere in your message to slip through the spam filter) | *Please contact Helen before application if you are interested in applying to the CSHL or SBU programs and work in our lab.</t>
+          <t>Please feel free to send an email to Arthur (see contact) to let him know to look out for your application.</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>Cheese3D (ML video analysis of facial movement) and the CSHL BioAI PhD program fit the applicant's interest in ML for biological/neural data (calcium imaging, EEG decoding).</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr"/>
+          <t>His interest in validating neural decoders (confounds, interpretability) connects to the EEG motor-imagery decoder with run-grouped validation.</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>psychology department; applications go through Psychology or Neuroscience program, not CS/Stats</t>
+        </is>
+      </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>dossier start_year: no snapshot, re-check</t>
+          <t>also listed as Arthur Sangil Lee</t>
         </is>
       </c>
     </row>
@@ -1033,22 +1037,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Duke University</t>
+          <t>Cold Spring Harbor Laboratory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mechanical Eng &amp; Materials Science; Center for Computational &amp; Digital Health Innovation</t>
+          <t>CSHL Faculty (Research)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Boyuan Chen</t>
+          <t>Helen Hou</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assistant Professor in the Thomas Lord Department of Mechanical Engineering and Mate</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1058,62 +1062,62 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>core-ML/CV</t>
+          <t>NeuroAI</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>12</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Trans. Mach. Learn. Res. 4, ICRA 3, CoRL 3, NeurIPS 1, IROS 1</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
-          <t>AI-type dept: Mechanical Eng &amp; Materials Science</t>
+          <t>check which PhD program can admit (not a CS/Stat/DS dept)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Robotics: learns realistic lip motions for humanoid face robots; physical AI.</t>
+          <t>Brain-body motor control; ML video analysis and neural encoding from behavior via Gaussian splatting.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>boyuan.chen@duke.edu</t>
+          <t>hou@cshl.edu</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>https://mems.duke.edu/people/boyuan-chen/</t>
+          <t>https://www.cshl.edu/research/faculty-staff/helen-hou/</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>http://generalroboticslab.com/</t>
+          <t>https://houlab.org</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ORCH: Organizational Principles Enable Collective Intelligence in Embodied AI</t>
+          <t>Cheese3D enables sensitive detection and analysis of whole-face movement in mice</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Online Sim-to-Real Adaptation via Closed-Loop System Modeling</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr"/>
+          <t>A generic noninvasive neuromotor interface for human-computer interaction</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>A case study on the use of end-to-end real-time monitoring to ensure quality of oral solid dosage forms in pharmaceutical development. (2025) | Chemical genetic screens reveal defective lysosomal trafficking as synthetic lethal with NF1 loss (2024)</t>
+        </is>
+      </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>https://mems.duke.edu/people?s=&amp;group=faculty-primary,faculty-secondary</t>
+          <t>https://www.cshl.edu/research/faculty-staff/</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1123,20 +1127,24 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unspecified: </t>
+          <t>Yes: We are actively recruiting at all levels, including but not limited to Students, Postdocs, and Research Technicians.</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>robotics, little overlap with applicant projects</t>
-        </is>
-      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Please get in touch via hou [at] cshl.edu and include your CV/resume and contact information of three references. (IMPORTANT: Please include the term #hou_lab _ candidate somewhere in your message to slip through the spam filter) | *Please contact Helen before application if you are interested in applying to the CSHL or SBU programs and work in our lab.</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Cheese3D (ML video analysis of facial movement) and the CSHL BioAI PhD program fit the applicant's interest in ML for biological/neural data (calcium imaging, EEG decoding).</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>dossier reader says B: Robotics / physical intelligence; AI-for-science pillar is a stretch for Bio-AI goal. Not A.</t>
+          <t>dossier start_year: no snapshot, re-check</t>
         </is>
       </c>
     </row>
@@ -1146,22 +1154,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>University of South Florida</t>
+          <t>Duke University</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bellini College of AI, Cybersecurity and Computing</t>
+          <t>Mechanical Eng &amp; Materials Science; Center for Computational &amp; Digital Health Innovation</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fengchun Qiao</t>
+          <t>Boyuan Chen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assistant Professor</t>
+          <t>Assistant Professor in the Thomas Lord Department of Mechanical Engineering and Mate</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1176,57 +1184,57 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>trustworthy-ML</t>
+          <t>core-ML/CV</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>ICML 2, CVPR 1, NeurIPS 1, ICLR 1, IEEE Trans. Pattern Anal. Mach. Intell. 1</t>
+          <t>Trans. Mach. Learn. Res. 4, ICRA 3, CoRL 3, NeurIPS 1, IROS 1</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>AI-type dept: Bellini College of AI, Cybersecurity and Comp</t>
+          <t>AI-type dept: Mechanical Eng &amp; Materials Science</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Trustworthy ML focused on out-of-distribution generalization, using robust optimization and graph theory.</t>
+          <t>Robotics: learns realistic lip motions for humanoid face robots; physical AI.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>fengchun@usf.edu</t>
+          <t>boyuan.chen@duke.edu</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/fengchun_qiao.aspx</t>
+          <t>https://mems.duke.edu/people/boyuan-chen/</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>https://joffery.github.io/joffery/</t>
+          <t>http://generalroboticslab.com/</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Structure-informed Risk Minimization for Robust Ensemble Learning</t>
+          <t>ORCH: Organizational Principles Enable Collective Intelligence in Embodied AI</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>SeafloorAI: A Large-scale Vision-Language Dataset for Seafloor Geological Survey</t>
+          <t>Online Sim-to-Real Adaptation via Closed-Loop System Modeling</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/index.aspx</t>
+          <t>https://mems.duke.edu/people?s=&amp;group=faculty-primary,faculty-secondary</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1241,13 +1249,17 @@
       </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Arborphy BioCLIP fusion with leakage-aware evaluation connects to OOD generalization / distribution-shift robustness.</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>robotics, little overlap with applicant projects</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>dossier reader says B: Robotics / physical intelligence; AI-for-science pillar is a stretch for Bio-AI goal. Not A.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1265,7 +1277,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Guangjing Wang</t>
+          <t>Fengchun Qiao</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1289,11 +1301,11 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>ACL (Findings) 1, ACL (1) 1, CVPR 1</t>
+          <t>ICML 2, CVPR 1, NeurIPS 1, ICLR 1, IEEE Trans. Pattern Anal. Mach. Intell. 1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1303,32 +1315,36 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Adaptive attacks on audio watermarking and speech spoofing detector benchmarks; also soil sensing system.</t>
+          <t>Trustworthy ML focused on out-of-distribution generalization, using robust optimization and graph theory.</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>guangjingwang@usf.edu</t>
+          <t>fengchun@usf.edu</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/guangjing-wang.aspx</t>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/fengchun_qiao.aspx</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/guangjing-wang.aspx</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>SoilNutri: A Passive Metasurface-based, Low-cost System for Soil Moisture and Nitrogen Monitoring (2026) | Learning to Evade: Adaptive Attacks on Audio Watermarking (2026)</t>
-        </is>
-      </c>
+          <t>https://joffery.github.io/joffery/</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Structure-informed Risk Minimization for Robust Ensemble Learning</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>SeafloorAI: A Large-scale Vision-Language Dataset for Seafloor Geological Survey</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
           <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/index.aspx</t>
@@ -1348,23 +1364,15 @@
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>multi-agent system with blind cross-model verification connects to his agentic-AI work.</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>no personal/lab site found after 2 searches; official page only</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>fit based on name-matched papers only: check they are this person's</t>
-        </is>
-      </c>
+          <t>Arborphy BioCLIP fusion with leakage-aware evaluation connects to OOD generalization / distribution-shift robustness.</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1373,12 +1381,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Electrical Engineering</t>
+          <t>Bellini College of AI, Cybersecurity and Computing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Xiaomin Lin</t>
+          <t>Guangjing Wang</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1398,61 +1406,53 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>core-ML/CV</t>
+          <t>trustworthy-ML</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>ICRA 4, IROS 3, WACV (Workshops) 1, AAAI 1, ECCV (65) 1</t>
+          <t>ACL (Findings) 1, ACL (1) 1, CVPR 1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>AI-type dept: Electrical Engineering</t>
+          <t>AI-type dept: Bellini College of AI, Cybersecurity and Comp</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Robotics, perception and edge AI for underwater and agricultural autonomy; deep learning rhino detection.</t>
+          <t>Adaptive attacks on audio watermarking and speech spoofing detector benchmarks; also soil sensing system.</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>xlin2@usf.edu</t>
+          <t>guangjingwang@usf.edu</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/engineering/ece/faculty-staff/lin-xiaomin.aspx</t>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/guangjing-wang.aspx</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>https://xiaominlin.github.io/</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>WaterGen</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>RAZOR</t>
-        </is>
-      </c>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/guangjing-wang.aspx</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Automated rhinoceros detection in satellite imagery using deep learning (2025) | A Kinodynamic Model for Dubins-Based Trajectory Planning in Precision Oyster Harvesting (2025)</t>
+          <t>SoilNutri: A Passive Metasurface-based, Low-cost System for Soil Moisture and Nitrogen Monitoring (2026) | Learning to Evade: Adaptive Attacks on Audio Watermarking (2026)</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>https://www.usf.edu/engineering/ece/faculty-staff/index.aspx</t>
+          <t>https://www.usf.edu/ai-cybersecurity-computing/people/faculty/index.aspx</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1462,22 +1462,26 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>Yes: I am actively recruiting PhD students to join my lab starting Spring 2027 and Fall 2027.</t>
+          <t xml:space="preserve">Unspecified: </t>
         </is>
       </c>
       <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Please read my Research Statement (PDF) before applying. | Competitive applicants typically hold an MS in a related field and have at least one top-tier publication. | Prospective students (not currently at USF) — fill out this application form . Please send an email to me as well, with your CV, transcripts, and a brief statement of your research interests and career goals. Tell me which of my papers or directions interest you and why. | You wrote the email yourself: Prospective Student - Bulls </t>
-        </is>
-      </c>
-      <c r="Y9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>multi-agent system with blind cross-model verification connects to his agentic-AI work.</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>site requires AI-disclosure tag (subject 'Prospective Student - Bulls 3Q') for AI-drafted emails; expects &gt;=1 top-tier publication (applicant has none); paper titles are only short names on homepage news (WaterGen ECCV 2026, RAZOR CVPR 2026 Findings)</t>
-        </is>
-      </c>
-      <c r="AA9" t="inlineStr"/>
+          <t>no personal/lab site found after 2 searches; official page only</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>fit based on name-matched papers only: check they are this person's</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1485,91 +1489,91 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Duke University</t>
+          <t>University of South Florida</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Electrical &amp; Computer Engineering</t>
+          <t>Electrical Engineering</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Neil Gong</t>
+          <t>Xiaomin Lin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Associate Professor of Electrical and Computer Engineering</t>
+          <t>Assistant Professor</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>associate</t>
+          <t>assistant</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>AI-for-science</t>
+          <t>core-ML/CV</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>NeurIPS 3, ICLR 2, ACL (1) 1, ACL (Findings) 1, EMNLP 1</t>
+          <t>ICRA 4, IROS 3, WACV (Workshops) 1, AAAI 1, ECCV (65) 1</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>AI-type dept: Electrical &amp; Computer Engineering</t>
+          <t>AI-type dept: Electrical Engineering</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Zero-shot autonomous microscopy for scalable characterization of 2D materials.</t>
+          <t>Robotics, perception and edge AI for underwater and agricultural autonomy; deep learning rhino detection.</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>neil.gong@duke.edu</t>
+          <t>xlin2@usf.edu</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>https://ece.duke.edu/people/neil-gong/</t>
+          <t>https://www.usf.edu/engineering/ece/faculty-staff/lin-xiaomin.aspx</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>https://people.duke.edu/~zg70/index.html</t>
+          <t>https://xiaominlin.github.io/</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>A Critical Evaluation of Defenses against Prompt Injection Attacks</t>
+          <t>WaterGen</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Fingerprinting LLMs via Prompt Injection</t>
+          <t>RAZOR</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Zero-Shot Autonomous Microscopy for Scalable and Intelligent Characterization of 2D Materials (2025)</t>
+          <t>Automated rhinoceros detection in satellite imagery using deep learning (2025) | A Kinodynamic Model for Dubins-Based Trajectory Planning in Precision Oyster Harvesting (2025)</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>https://ece.duke.edu/faculty</t>
+          <t>https://www.usf.edu/engineering/ece/faculty-staff/index.aspx</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1579,26 +1583,22 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>Yes: I am looking for postdocs, Ph.D. students, master's students, and undergraduate researchers. If you are interested in pursuing a Ph.D., please submit your application to Duke ECE.</t>
+          <t>Yes: I am actively recruiting PhD students to join my lab starting Spring 2027 and Fall 2027.</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>His work on evaluating prompt-injection defenses and secure agentic AI connects to my multi-agent system with verification and trust gating (agents).</t>
-        </is>
-      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Please read my Research Statement (PDF) before applying. | Competitive applicants typically hold an MS in a related field and have at least one top-tier publication. | Prospective students (not currently at USF) — fill out this application form . Please send an email to me as well, with your CV, transcripts, and a brief statement of your research interests and career goals. Tell me which of my papers or directions interest you and why. | You wrote the email yourself: Prospective Student - Bulls </t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>first-pass summary describes different work (microscopy of 2D materials); possibly wrong person/mismatch; warns he receives many emails and may not respond</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>associate: confirm promoted 2020+; fit based on name-matched papers only: check they are this person's</t>
-        </is>
-      </c>
+          <t>site requires AI-disclosure tag (subject 'Prospective Student - Bulls 3Q') for AI-drafted emails; expects &gt;=1 top-tier publication (applicant has none); paper titles are only short names on homepage news (WaterGen ECCV 2026, RAZOR CVPR 2026 Findings)</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">

</xml_diff>